<commit_message>
slow but steady progress on the plots
</commit_message>
<xml_diff>
--- a/data/Data Dictionary.xlsx
+++ b/data/Data Dictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stepheaneff/Documents/work/costed-NAPHS/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46773C05-2007-4046-A505-3F96EDB7B826}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BA4482F-BD35-ED4D-8B9E-1370386791DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="100" yWindow="760" windowWidth="29780" windowHeight="16820" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="100" yWindow="760" windowWidth="29780" windowHeight="16820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table information" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="248">
   <si>
     <t>Text</t>
   </si>
@@ -604,9 +604,6 @@
   </si>
   <si>
     <t>Steph Eaneff</t>
-  </si>
-  <si>
-    <t>The data dictionary was last updated on 23 April, 2025</t>
   </si>
   <si>
     <t>Raw Costed NAPHS data</t>
@@ -761,6 +758,30 @@
   </si>
   <si>
     <t>The estimated cost, standardized to USD (2024). Data were first converted into USD based on published exchange rates of of December of the specified year, then inflation-adjusted based on the CPI to USD (2024).</t>
+  </si>
+  <si>
+    <t>24 April, 2025</t>
+  </si>
+  <si>
+    <t>Update coding of Liberia core capacity to correctly reflect core capacity "Medical Countermeasures" instead of IPC</t>
+  </si>
+  <si>
+    <t>Liberia Costed NAPHS</t>
+  </si>
+  <si>
+    <t>The data dictionary was last updated on 24 April, 2025</t>
+  </si>
+  <si>
+    <t>Requirement highlights</t>
+  </si>
+  <si>
+    <t>For plots and specific analysis, brief summary statements of specific requirements documented in the file Clean Costed NAPHS data and Raw Costed NAPHS data, interim file created by research team for the purpose of generating figures</t>
+  </si>
+  <si>
+    <t>one row per desired label on a plot</t>
+  </si>
+  <si>
+    <t>Generated by research team</t>
   </si>
 </sst>
 </file>
@@ -1022,27 +1043,6 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1057,9 +1057,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1081,6 +1078,30 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1321,42 +1342,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="16"/>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
+      <c r="A1" s="29"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
     </row>
     <row r="2" spans="1:22" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="32" t="s">
         <v>147</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
     </row>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="30" t="s">
         <v>148</v>
       </c>
-      <c r="B3" s="18"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
+      <c r="B3" s="31"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
     </row>
     <row r="4" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="18" t="s">
-        <v>189</v>
-      </c>
-      <c r="B4" s="18"/>
-      <c r="C4" s="18"/>
-      <c r="D4" s="18"/>
+      <c r="A4" s="31" t="s">
+        <v>243</v>
+      </c>
+      <c r="B4" s="31"/>
+      <c r="C4" s="31"/>
+      <c r="D4" s="31"/>
     </row>
     <row r="5" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="31" t="s">
         <v>149</v>
       </c>
-      <c r="B5" s="18"/>
-      <c r="C5" s="18"/>
-      <c r="D5" s="18"/>
+      <c r="B5" s="31"/>
+      <c r="C5" s="31"/>
+      <c r="D5" s="31"/>
     </row>
     <row r="6" spans="1:22" ht="17" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6"/>
@@ -1365,13 +1386,13 @@
       <c r="D6" s="6"/>
     </row>
     <row r="7" spans="1:22" ht="37" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="28" t="s">
         <v>132</v>
       </c>
-      <c r="B7" s="15"/>
-      <c r="C7" s="15"/>
-      <c r="D7" s="15"/>
-      <c r="E7" s="15"/>
+      <c r="B7" s="28"/>
+      <c r="C7" s="28"/>
+      <c r="D7" s="28"/>
+      <c r="E7" s="28"/>
     </row>
     <row r="8" spans="1:22" ht="32.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A8" s="12" t="s">
@@ -1391,28 +1412,28 @@
       </c>
     </row>
     <row r="9" spans="1:22" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="14" t="s">
-        <v>193</v>
-      </c>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
+      <c r="A9" s="26" t="s">
+        <v>192</v>
+      </c>
+      <c r="B9" s="26"/>
+      <c r="C9" s="26"/>
+      <c r="D9" s="26"/>
+      <c r="E9" s="26"/>
     </row>
     <row r="10" spans="1:22" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="22" t="s">
+      <c r="A10" s="15" t="s">
         <v>150</v>
       </c>
-      <c r="B10" s="22" t="s">
+      <c r="B10" s="15" t="s">
         <v>154</v>
       </c>
-      <c r="C10" s="22" t="s">
+      <c r="C10" s="15" t="s">
         <v>153</v>
       </c>
-      <c r="D10" s="22" t="s">
+      <c r="D10" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="E10" s="22" t="s">
+      <c r="E10" s="15" t="s">
         <v>155</v>
       </c>
       <c r="F10" s="2"/>
@@ -1434,13 +1455,13 @@
       <c r="V10" s="2"/>
     </row>
     <row r="11" spans="1:22" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="26" t="s">
-        <v>194</v>
-      </c>
-      <c r="B11" s="26"/>
-      <c r="C11" s="26"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26"/>
+      <c r="A11" s="27" t="s">
+        <v>193</v>
+      </c>
+      <c r="B11" s="27"/>
+      <c r="C11" s="27"/>
+      <c r="D11" s="27"/>
+      <c r="E11" s="27"/>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
@@ -1460,19 +1481,19 @@
       <c r="V11" s="2"/>
     </row>
     <row r="12" spans="1:22" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="22" t="s">
-        <v>190</v>
-      </c>
-      <c r="B12" s="22" t="s">
-        <v>192</v>
-      </c>
-      <c r="C12" s="22" t="s">
+      <c r="A12" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="B12" s="15" t="s">
+        <v>191</v>
+      </c>
+      <c r="C12" s="15" t="s">
         <v>153</v>
       </c>
-      <c r="D12" s="22" t="s">
+      <c r="D12" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="E12" s="22" t="s">
+      <c r="E12" s="15" t="s">
         <v>155</v>
       </c>
       <c r="F12" s="2"/>
@@ -1494,19 +1515,19 @@
       <c r="V12" s="2"/>
     </row>
     <row r="13" spans="1:22" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="23" t="s">
-        <v>197</v>
-      </c>
-      <c r="B13" s="24" t="s">
+      <c r="A13" s="16" t="s">
+        <v>196</v>
+      </c>
+      <c r="B13" s="17" t="s">
+        <v>210</v>
+      </c>
+      <c r="C13" s="16" t="s">
         <v>211</v>
       </c>
-      <c r="C13" s="23" t="s">
-        <v>212</v>
-      </c>
-      <c r="D13" s="23" t="s">
+      <c r="D13" s="16" t="s">
         <v>151</v>
       </c>
-      <c r="E13" s="22" t="s">
+      <c r="E13" s="15" t="s">
         <v>155</v>
       </c>
       <c r="F13" s="2"/>
@@ -1528,20 +1549,20 @@
       <c r="V13" s="2"/>
     </row>
     <row r="14" spans="1:22" ht="97" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="22" t="s">
+      <c r="A14" s="15" t="s">
+        <v>212</v>
+      </c>
+      <c r="B14" s="18" t="s">
         <v>213</v>
       </c>
-      <c r="B14" s="25" t="s">
+      <c r="C14" s="15" t="s">
         <v>214</v>
       </c>
-      <c r="C14" s="22" t="s">
+      <c r="D14" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="E14" s="15" t="s">
         <v>215</v>
-      </c>
-      <c r="D14" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="E14" s="22" t="s">
-        <v>216</v>
       </c>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
@@ -1561,12 +1582,22 @@
       <c r="U14" s="2"/>
       <c r="V14" s="2"/>
     </row>
-    <row r="15" spans="1:22" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="7"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="2"/>
+    <row r="15" spans="1:22" ht="63" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="15" t="s">
+        <v>244</v>
+      </c>
+      <c r="B15" s="18" t="s">
+        <v>245</v>
+      </c>
+      <c r="C15" s="15" t="s">
+        <v>246</v>
+      </c>
+      <c r="D15" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="E15" s="15" t="s">
+        <v>247</v>
+      </c>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
@@ -3628,14 +3659,14 @@
       <c r="D1" s="6"/>
     </row>
     <row r="2" spans="1:21" ht="37" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="28" t="s">
         <v>136</v>
       </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
     </row>
     <row r="3" spans="1:21" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A3" s="12" t="s">
@@ -3658,32 +3689,32 @@
       </c>
     </row>
     <row r="4" spans="1:21" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="14" t="s">
-        <v>195</v>
-      </c>
-      <c r="B4" s="14"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
+      <c r="A4" s="26" t="s">
+        <v>194</v>
+      </c>
+      <c r="B4" s="26"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
     </row>
     <row r="5" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="15" t="s">
         <v>150</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="15" t="s">
         <v>174</v>
       </c>
-      <c r="C5" s="22" t="s">
+      <c r="C5" s="15" t="s">
         <v>156</v>
       </c>
-      <c r="D5" s="22" t="s">
+      <c r="D5" s="15" t="s">
         <v>165</v>
       </c>
-      <c r="E5" s="22" t="s">
+      <c r="E5" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="F5" s="22" t="s">
+      <c r="F5" s="15" t="s">
         <v>186</v>
       </c>
       <c r="G5" s="2"/>
@@ -3703,23 +3734,23 @@
       <c r="U5" s="2"/>
     </row>
     <row r="6" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="15" t="s">
         <v>150</v>
       </c>
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="15" t="s">
+        <v>197</v>
+      </c>
+      <c r="C6" s="15" t="s">
         <v>198</v>
       </c>
-      <c r="C6" s="22" t="s">
-        <v>199</v>
-      </c>
-      <c r="D6" s="27" t="s">
+      <c r="D6" s="19" t="s">
+        <v>208</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>183</v>
+      </c>
+      <c r="F6" s="20" t="s">
         <v>209</v>
-      </c>
-      <c r="E6" s="22" t="s">
-        <v>183</v>
-      </c>
-      <c r="F6" s="28" t="s">
-        <v>210</v>
       </c>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
@@ -3738,22 +3769,22 @@
       <c r="U6" s="2"/>
     </row>
     <row r="7" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="15" t="s">
         <v>150</v>
       </c>
-      <c r="B7" s="25" t="s">
+      <c r="B7" s="18" t="s">
         <v>175</v>
       </c>
-      <c r="C7" s="25" t="s">
+      <c r="C7" s="18" t="s">
         <v>157</v>
       </c>
-      <c r="D7" s="27" t="s">
-        <v>208</v>
-      </c>
-      <c r="E7" s="22" t="s">
+      <c r="D7" s="19" t="s">
+        <v>207</v>
+      </c>
+      <c r="E7" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="F7" s="22" t="s">
+      <c r="F7" s="15" t="s">
         <v>186</v>
       </c>
       <c r="G7" s="2"/>
@@ -3773,22 +3804,22 @@
       <c r="U7" s="2"/>
     </row>
     <row r="8" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="22" t="s">
+      <c r="A8" s="15" t="s">
         <v>150</v>
       </c>
-      <c r="B8" s="25" t="s">
+      <c r="B8" s="18" t="s">
         <v>176</v>
       </c>
-      <c r="C8" s="22" t="s">
+      <c r="C8" s="15" t="s">
         <v>158</v>
       </c>
-      <c r="D8" s="27" t="s">
+      <c r="D8" s="19" t="s">
         <v>167</v>
       </c>
-      <c r="E8" s="22" t="s">
+      <c r="E8" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="F8" s="22" t="s">
+      <c r="F8" s="15" t="s">
         <v>186</v>
       </c>
       <c r="G8" s="2"/>
@@ -3808,22 +3839,22 @@
       <c r="U8" s="2"/>
     </row>
     <row r="9" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="22" t="s">
+      <c r="A9" s="15" t="s">
         <v>150</v>
       </c>
-      <c r="B9" s="25" t="s">
+      <c r="B9" s="18" t="s">
         <v>177</v>
       </c>
-      <c r="C9" s="22" t="s">
+      <c r="C9" s="15" t="s">
         <v>159</v>
       </c>
-      <c r="D9" s="27" t="s">
+      <c r="D9" s="19" t="s">
         <v>168</v>
       </c>
-      <c r="E9" s="22" t="s">
+      <c r="E9" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="F9" s="22" t="s">
+      <c r="F9" s="15" t="s">
         <v>186</v>
       </c>
       <c r="G9" s="2"/>
@@ -3843,22 +3874,22 @@
       <c r="U9" s="2"/>
     </row>
     <row r="10" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="22" t="s">
+      <c r="A10" s="15" t="s">
         <v>150</v>
       </c>
-      <c r="B10" s="25" t="s">
+      <c r="B10" s="18" t="s">
         <v>178</v>
       </c>
-      <c r="C10" s="22" t="s">
+      <c r="C10" s="15" t="s">
         <v>160</v>
       </c>
-      <c r="D10" s="22" t="s">
+      <c r="D10" s="15" t="s">
         <v>169</v>
       </c>
-      <c r="E10" s="22" t="s">
+      <c r="E10" s="15" t="s">
         <v>184</v>
       </c>
-      <c r="F10" s="22" t="s">
+      <c r="F10" s="15" t="s">
         <v>186</v>
       </c>
       <c r="G10" s="2"/>
@@ -3878,22 +3909,22 @@
       <c r="U10" s="2"/>
     </row>
     <row r="11" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="15" t="s">
         <v>150</v>
       </c>
-      <c r="B11" s="25" t="s">
+      <c r="B11" s="18" t="s">
         <v>179</v>
       </c>
-      <c r="C11" s="25" t="s">
+      <c r="C11" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="D11" s="22" t="s">
+      <c r="D11" s="15" t="s">
         <v>170</v>
       </c>
-      <c r="E11" s="22" t="s">
+      <c r="E11" s="15" t="s">
         <v>184</v>
       </c>
-      <c r="F11" s="22" t="s">
+      <c r="F11" s="15" t="s">
         <v>186</v>
       </c>
       <c r="G11" s="2"/>
@@ -3913,22 +3944,22 @@
       <c r="U11" s="2"/>
     </row>
     <row r="12" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="22" t="s">
+      <c r="A12" s="15" t="s">
         <v>150</v>
       </c>
-      <c r="B12" s="25" t="s">
+      <c r="B12" s="18" t="s">
+        <v>233</v>
+      </c>
+      <c r="C12" s="18" t="s">
         <v>234</v>
       </c>
-      <c r="C12" s="25" t="s">
+      <c r="D12" s="15" t="s">
         <v>235</v>
       </c>
-      <c r="D12" s="22" t="s">
-        <v>236</v>
-      </c>
-      <c r="E12" s="22" t="s">
+      <c r="E12" s="15" t="s">
         <v>185</v>
       </c>
-      <c r="F12" s="22" t="s">
+      <c r="F12" s="15" t="s">
         <v>186</v>
       </c>
       <c r="G12" s="2"/>
@@ -3948,22 +3979,22 @@
       <c r="U12" s="2"/>
     </row>
     <row r="13" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="22" t="s">
+      <c r="A13" s="15" t="s">
         <v>150</v>
       </c>
-      <c r="B13" s="25" t="s">
-        <v>217</v>
-      </c>
-      <c r="C13" s="25" t="s">
-        <v>222</v>
-      </c>
-      <c r="D13" s="22" t="s">
-        <v>237</v>
-      </c>
-      <c r="E13" s="22" t="s">
+      <c r="B13" s="18" t="s">
+        <v>216</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>221</v>
+      </c>
+      <c r="D13" s="15" t="s">
+        <v>236</v>
+      </c>
+      <c r="E13" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="F13" s="22" t="s">
+      <c r="F13" s="15" t="s">
         <v>186</v>
       </c>
       <c r="G13" s="2"/>
@@ -3983,23 +4014,23 @@
       <c r="U13" s="2"/>
     </row>
     <row r="14" spans="1:21" ht="84" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="22" t="s">
+      <c r="A14" s="15" t="s">
         <v>150</v>
       </c>
-      <c r="B14" s="25" t="s">
+      <c r="B14" s="18" t="s">
+        <v>237</v>
+      </c>
+      <c r="C14" s="18" t="s">
         <v>238</v>
       </c>
-      <c r="C14" s="25" t="s">
+      <c r="D14" s="15" t="s">
         <v>239</v>
       </c>
-      <c r="D14" s="22" t="s">
-        <v>240</v>
-      </c>
-      <c r="E14" s="22" t="s">
+      <c r="E14" s="15" t="s">
         <v>185</v>
       </c>
-      <c r="F14" s="22" t="s">
-        <v>216</v>
+      <c r="F14" s="15" t="s">
+        <v>215</v>
       </c>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
@@ -4018,22 +4049,22 @@
       <c r="U14" s="2"/>
     </row>
     <row r="15" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="22" t="s">
+      <c r="A15" s="15" t="s">
         <v>150</v>
       </c>
-      <c r="B15" s="22" t="s">
+      <c r="B15" s="15" t="s">
         <v>182</v>
       </c>
-      <c r="C15" s="25" t="s">
+      <c r="C15" s="18" t="s">
         <v>164</v>
       </c>
-      <c r="D15" s="22" t="s">
+      <c r="D15" s="15" t="s">
         <v>173</v>
       </c>
-      <c r="E15" s="22" t="s">
+      <c r="E15" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="F15" s="22" t="s">
+      <c r="F15" s="15" t="s">
         <v>186</v>
       </c>
       <c r="G15" s="2"/>
@@ -4053,32 +4084,32 @@
       <c r="U15" s="2"/>
     </row>
     <row r="16" spans="1:21" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="26" t="s">
-        <v>196</v>
-      </c>
-      <c r="B16" s="26"/>
-      <c r="C16" s="26"/>
-      <c r="D16" s="26"/>
-      <c r="E16" s="26"/>
-      <c r="F16" s="26"/>
+      <c r="A16" s="27" t="s">
+        <v>195</v>
+      </c>
+      <c r="B16" s="27"/>
+      <c r="C16" s="27"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="27"/>
+      <c r="F16" s="27"/>
     </row>
     <row r="17" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="22" t="s">
-        <v>190</v>
-      </c>
-      <c r="B17" s="22" t="s">
+      <c r="A17" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="B17" s="15" t="s">
         <v>174</v>
       </c>
-      <c r="C17" s="22" t="s">
+      <c r="C17" s="15" t="s">
         <v>156</v>
       </c>
-      <c r="D17" s="22" t="s">
+      <c r="D17" s="15" t="s">
         <v>165</v>
       </c>
-      <c r="E17" s="22" t="s">
+      <c r="E17" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="F17" s="22" t="s">
+      <c r="F17" s="15" t="s">
         <v>186</v>
       </c>
       <c r="G17" s="2"/>
@@ -4098,22 +4129,22 @@
       <c r="U17" s="2"/>
     </row>
     <row r="18" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="22" t="s">
-        <v>190</v>
-      </c>
-      <c r="B18" s="25" t="s">
+      <c r="A18" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="B18" s="18" t="s">
         <v>175</v>
       </c>
-      <c r="C18" s="25" t="s">
+      <c r="C18" s="18" t="s">
         <v>157</v>
       </c>
-      <c r="D18" s="27" t="s">
+      <c r="D18" s="19" t="s">
         <v>166</v>
       </c>
-      <c r="E18" s="22" t="s">
+      <c r="E18" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="F18" s="22" t="s">
+      <c r="F18" s="15" t="s">
         <v>186</v>
       </c>
       <c r="G18" s="2"/>
@@ -4133,22 +4164,22 @@
       <c r="U18" s="2"/>
     </row>
     <row r="19" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="22" t="s">
-        <v>190</v>
-      </c>
-      <c r="B19" s="25" t="s">
+      <c r="A19" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="B19" s="18" t="s">
         <v>176</v>
       </c>
-      <c r="C19" s="22" t="s">
+      <c r="C19" s="15" t="s">
         <v>158</v>
       </c>
-      <c r="D19" s="27" t="s">
+      <c r="D19" s="19" t="s">
         <v>167</v>
       </c>
-      <c r="E19" s="22" t="s">
+      <c r="E19" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="F19" s="22" t="s">
+      <c r="F19" s="15" t="s">
         <v>186</v>
       </c>
       <c r="G19" s="2"/>
@@ -4168,22 +4199,22 @@
       <c r="U19" s="2"/>
     </row>
     <row r="20" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="22" t="s">
-        <v>190</v>
-      </c>
-      <c r="B20" s="25" t="s">
+      <c r="A20" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="B20" s="18" t="s">
         <v>177</v>
       </c>
-      <c r="C20" s="22" t="s">
+      <c r="C20" s="15" t="s">
         <v>159</v>
       </c>
-      <c r="D20" s="27" t="s">
+      <c r="D20" s="19" t="s">
         <v>168</v>
       </c>
-      <c r="E20" s="22" t="s">
+      <c r="E20" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="F20" s="22" t="s">
+      <c r="F20" s="15" t="s">
         <v>186</v>
       </c>
       <c r="G20" s="2"/>
@@ -4203,22 +4234,22 @@
       <c r="U20" s="2"/>
     </row>
     <row r="21" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="22" t="s">
-        <v>190</v>
-      </c>
-      <c r="B21" s="25" t="s">
+      <c r="A21" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="B21" s="18" t="s">
         <v>178</v>
       </c>
-      <c r="C21" s="22" t="s">
+      <c r="C21" s="15" t="s">
         <v>160</v>
       </c>
-      <c r="D21" s="22" t="s">
+      <c r="D21" s="15" t="s">
         <v>169</v>
       </c>
-      <c r="E21" s="22" t="s">
+      <c r="E21" s="15" t="s">
         <v>184</v>
       </c>
-      <c r="F21" s="22" t="s">
+      <c r="F21" s="15" t="s">
         <v>186</v>
       </c>
       <c r="G21" s="2"/>
@@ -4238,22 +4269,22 @@
       <c r="U21" s="2"/>
     </row>
     <row r="22" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="22" t="s">
-        <v>190</v>
-      </c>
-      <c r="B22" s="25" t="s">
+      <c r="A22" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="B22" s="18" t="s">
         <v>179</v>
       </c>
-      <c r="C22" s="25" t="s">
+      <c r="C22" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="D22" s="22" t="s">
+      <c r="D22" s="15" t="s">
         <v>170</v>
       </c>
-      <c r="E22" s="22" t="s">
+      <c r="E22" s="15" t="s">
         <v>184</v>
       </c>
-      <c r="F22" s="22" t="s">
+      <c r="F22" s="15" t="s">
         <v>186</v>
       </c>
       <c r="G22" s="2"/>
@@ -4273,22 +4304,22 @@
       <c r="U22" s="2"/>
     </row>
     <row r="23" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="22" t="s">
-        <v>190</v>
-      </c>
-      <c r="B23" s="25" t="s">
+      <c r="A23" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="B23" s="18" t="s">
         <v>180</v>
       </c>
-      <c r="C23" s="25" t="s">
+      <c r="C23" s="18" t="s">
         <v>162</v>
       </c>
-      <c r="D23" s="22" t="s">
+      <c r="D23" s="15" t="s">
         <v>171</v>
       </c>
-      <c r="E23" s="22" t="s">
+      <c r="E23" s="15" t="s">
         <v>185</v>
       </c>
-      <c r="F23" s="22" t="s">
+      <c r="F23" s="15" t="s">
         <v>186</v>
       </c>
       <c r="G23" s="2"/>
@@ -4308,22 +4339,22 @@
       <c r="U23" s="2"/>
     </row>
     <row r="24" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="22" t="s">
-        <v>190</v>
-      </c>
-      <c r="B24" s="25" t="s">
+      <c r="A24" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="B24" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="C24" s="25" t="s">
+      <c r="C24" s="18" t="s">
         <v>163</v>
       </c>
-      <c r="D24" s="22" t="s">
+      <c r="D24" s="15" t="s">
         <v>172</v>
       </c>
-      <c r="E24" s="22" t="s">
+      <c r="E24" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="F24" s="22" t="s">
+      <c r="F24" s="15" t="s">
         <v>186</v>
       </c>
       <c r="G24" s="2"/>
@@ -4343,22 +4374,22 @@
       <c r="U24" s="2"/>
     </row>
     <row r="25" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="22" t="s">
-        <v>190</v>
-      </c>
-      <c r="B25" s="22" t="s">
+      <c r="A25" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="B25" s="15" t="s">
         <v>182</v>
       </c>
-      <c r="C25" s="25" t="s">
+      <c r="C25" s="18" t="s">
         <v>164</v>
       </c>
-      <c r="D25" s="22" t="s">
+      <c r="D25" s="15" t="s">
         <v>173</v>
       </c>
-      <c r="E25" s="22" t="s">
+      <c r="E25" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="F25" s="22" t="s">
+      <c r="F25" s="15" t="s">
         <v>186</v>
       </c>
       <c r="G25" s="2"/>
@@ -4378,23 +4409,23 @@
       <c r="U25" s="2"/>
     </row>
     <row r="26" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="22" t="s">
+      <c r="A26" s="15" t="s">
+        <v>196</v>
+      </c>
+      <c r="B26" s="15" t="s">
         <v>197</v>
       </c>
-      <c r="B26" s="22" t="s">
+      <c r="C26" s="15" t="s">
         <v>198</v>
       </c>
-      <c r="C26" s="22" t="s">
-        <v>199</v>
-      </c>
-      <c r="D26" s="29" t="s">
-        <v>204</v>
-      </c>
-      <c r="E26" s="22" t="s">
+      <c r="D26" s="21" t="s">
+        <v>203</v>
+      </c>
+      <c r="E26" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="F26" s="29" t="s">
-        <v>207</v>
+      <c r="F26" s="21" t="s">
+        <v>206</v>
       </c>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
@@ -4413,23 +4444,23 @@
       <c r="U26" s="2"/>
     </row>
     <row r="27" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="22" t="s">
-        <v>197</v>
-      </c>
-      <c r="B27" s="22" t="s">
-        <v>200</v>
-      </c>
-      <c r="C27" s="22" t="s">
-        <v>202</v>
-      </c>
-      <c r="D27" s="29" t="s">
-        <v>205</v>
-      </c>
-      <c r="E27" s="22" t="s">
+      <c r="A27" s="15" t="s">
+        <v>196</v>
+      </c>
+      <c r="B27" s="15" t="s">
+        <v>199</v>
+      </c>
+      <c r="C27" s="15" t="s">
+        <v>201</v>
+      </c>
+      <c r="D27" s="21" t="s">
+        <v>204</v>
+      </c>
+      <c r="E27" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="F27" s="29" t="s">
-        <v>207</v>
+      <c r="F27" s="21" t="s">
+        <v>206</v>
       </c>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
@@ -4448,23 +4479,23 @@
       <c r="U27" s="2"/>
     </row>
     <row r="28" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="22" t="s">
-        <v>197</v>
-      </c>
-      <c r="B28" s="22" t="s">
-        <v>201</v>
-      </c>
-      <c r="C28" s="22" t="s">
-        <v>203</v>
-      </c>
-      <c r="D28" s="29" t="s">
+      <c r="A28" s="15" t="s">
+        <v>196</v>
+      </c>
+      <c r="B28" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="C28" s="15" t="s">
+        <v>202</v>
+      </c>
+      <c r="D28" s="21" t="s">
+        <v>205</v>
+      </c>
+      <c r="E28" s="15" t="s">
+        <v>183</v>
+      </c>
+      <c r="F28" s="21" t="s">
         <v>206</v>
-      </c>
-      <c r="E28" s="22" t="s">
-        <v>183</v>
-      </c>
-      <c r="F28" s="29" t="s">
-        <v>207</v>
       </c>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
@@ -4483,23 +4514,23 @@
       <c r="U28" s="2"/>
     </row>
     <row r="29" spans="1:21" ht="84" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="22" t="s">
-        <v>213</v>
-      </c>
-      <c r="B29" s="22" t="s">
-        <v>217</v>
-      </c>
-      <c r="C29" s="22" t="s">
-        <v>222</v>
-      </c>
-      <c r="D29" s="29" t="s">
-        <v>227</v>
-      </c>
-      <c r="E29" s="22" t="s">
+      <c r="A29" s="15" t="s">
+        <v>212</v>
+      </c>
+      <c r="B29" s="15" t="s">
+        <v>216</v>
+      </c>
+      <c r="C29" s="15" t="s">
+        <v>221</v>
+      </c>
+      <c r="D29" s="21" t="s">
+        <v>226</v>
+      </c>
+      <c r="E29" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="F29" s="22" t="s">
-        <v>216</v>
+      <c r="F29" s="15" t="s">
+        <v>215</v>
       </c>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
@@ -4518,23 +4549,23 @@
       <c r="U29" s="2"/>
     </row>
     <row r="30" spans="1:21" ht="82" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="22" t="s">
-        <v>213</v>
-      </c>
-      <c r="B30" s="22" t="s">
-        <v>218</v>
-      </c>
-      <c r="C30" s="22" t="s">
-        <v>223</v>
-      </c>
-      <c r="D30" s="22" t="s">
-        <v>228</v>
-      </c>
-      <c r="E30" s="22" t="s">
+      <c r="A30" s="15" t="s">
+        <v>212</v>
+      </c>
+      <c r="B30" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="C30" s="15" t="s">
+        <v>222</v>
+      </c>
+      <c r="D30" s="15" t="s">
+        <v>227</v>
+      </c>
+      <c r="E30" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="F30" s="22" t="s">
-        <v>216</v>
+      <c r="F30" s="15" t="s">
+        <v>215</v>
       </c>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
@@ -4553,23 +4584,23 @@
       <c r="U30" s="2"/>
     </row>
     <row r="31" spans="1:21" ht="82" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="22" t="s">
-        <v>213</v>
-      </c>
-      <c r="B31" s="22" t="s">
-        <v>219</v>
-      </c>
-      <c r="C31" s="22" t="s">
-        <v>224</v>
-      </c>
-      <c r="D31" s="22" t="s">
-        <v>229</v>
-      </c>
-      <c r="E31" s="22" t="s">
+      <c r="A31" s="15" t="s">
+        <v>212</v>
+      </c>
+      <c r="B31" s="15" t="s">
+        <v>218</v>
+      </c>
+      <c r="C31" s="15" t="s">
+        <v>223</v>
+      </c>
+      <c r="D31" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="E31" s="15" t="s">
         <v>185</v>
       </c>
-      <c r="F31" s="22" t="s">
-        <v>216</v>
+      <c r="F31" s="15" t="s">
+        <v>215</v>
       </c>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
@@ -4588,23 +4619,23 @@
       <c r="U31" s="2"/>
     </row>
     <row r="32" spans="1:21" ht="83" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="22" t="s">
-        <v>213</v>
-      </c>
-      <c r="B32" s="22" t="s">
-        <v>220</v>
-      </c>
-      <c r="C32" s="22" t="s">
-        <v>225</v>
-      </c>
-      <c r="D32" s="22" t="s">
-        <v>230</v>
-      </c>
-      <c r="E32" s="22" t="s">
+      <c r="A32" s="15" t="s">
+        <v>212</v>
+      </c>
+      <c r="B32" s="15" t="s">
+        <v>219</v>
+      </c>
+      <c r="C32" s="15" t="s">
+        <v>224</v>
+      </c>
+      <c r="D32" s="15" t="s">
+        <v>229</v>
+      </c>
+      <c r="E32" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="F32" s="22" t="s">
-        <v>216</v>
+      <c r="F32" s="15" t="s">
+        <v>215</v>
       </c>
       <c r="G32" s="2"/>
       <c r="H32" s="2"/>
@@ -4623,23 +4654,23 @@
       <c r="U32" s="2"/>
     </row>
     <row r="33" spans="1:21" ht="83" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="22" t="s">
-        <v>213</v>
-      </c>
-      <c r="B33" s="22" t="s">
-        <v>221</v>
-      </c>
-      <c r="C33" s="22" t="s">
-        <v>226</v>
-      </c>
-      <c r="D33" s="22" t="s">
-        <v>231</v>
-      </c>
-      <c r="E33" s="22" t="s">
+      <c r="A33" s="15" t="s">
+        <v>212</v>
+      </c>
+      <c r="B33" s="15" t="s">
+        <v>220</v>
+      </c>
+      <c r="C33" s="15" t="s">
+        <v>225</v>
+      </c>
+      <c r="D33" s="15" t="s">
+        <v>230</v>
+      </c>
+      <c r="E33" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="F33" s="22" t="s">
-        <v>216</v>
+      <c r="F33" s="15" t="s">
+        <v>215</v>
       </c>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
@@ -4662,8 +4693,8 @@
       <c r="B34" s="11"/>
       <c r="C34" s="11"/>
       <c r="D34" s="11"/>
-      <c r="E34" s="21"/>
-      <c r="F34" s="21"/>
+      <c r="E34" s="14"/>
+      <c r="F34" s="14"/>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
       <c r="I34" s="2"/>
@@ -4685,8 +4716,8 @@
       <c r="B35" s="11"/>
       <c r="C35" s="11"/>
       <c r="D35" s="11"/>
-      <c r="E35" s="21"/>
-      <c r="F35" s="21"/>
+      <c r="E35" s="14"/>
+      <c r="F35" s="14"/>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="2"/>
@@ -4708,8 +4739,8 @@
       <c r="B36" s="11"/>
       <c r="C36" s="11"/>
       <c r="D36" s="11"/>
-      <c r="E36" s="21"/>
-      <c r="F36" s="21"/>
+      <c r="E36" s="14"/>
+      <c r="F36" s="14"/>
       <c r="G36" s="3"/>
       <c r="H36" s="3"/>
       <c r="I36" s="3"/>
@@ -4731,8 +4762,8 @@
       <c r="B37" s="11"/>
       <c r="C37" s="11"/>
       <c r="D37" s="11"/>
-      <c r="E37" s="21"/>
-      <c r="F37" s="21"/>
+      <c r="E37" s="14"/>
+      <c r="F37" s="14"/>
       <c r="G37" s="3"/>
       <c r="H37" s="3"/>
       <c r="I37" s="3"/>
@@ -4754,8 +4785,8 @@
       <c r="B38" s="11"/>
       <c r="C38" s="11"/>
       <c r="D38" s="11"/>
-      <c r="E38" s="21"/>
-      <c r="F38" s="21"/>
+      <c r="E38" s="14"/>
+      <c r="F38" s="14"/>
       <c r="G38" s="3"/>
       <c r="H38" s="3"/>
       <c r="I38" s="3"/>
@@ -4777,8 +4808,8 @@
       <c r="B39" s="11"/>
       <c r="C39" s="11"/>
       <c r="D39" s="11"/>
-      <c r="E39" s="21"/>
-      <c r="F39" s="21"/>
+      <c r="E39" s="14"/>
+      <c r="F39" s="14"/>
       <c r="G39" s="3"/>
       <c r="H39" s="3"/>
       <c r="I39" s="3"/>
@@ -4800,8 +4831,8 @@
       <c r="B40" s="11"/>
       <c r="C40" s="11"/>
       <c r="D40" s="11"/>
-      <c r="E40" s="21"/>
-      <c r="F40" s="21"/>
+      <c r="E40" s="14"/>
+      <c r="F40" s="14"/>
       <c r="G40" s="3"/>
       <c r="H40" s="3"/>
       <c r="I40" s="3"/>
@@ -4819,12 +4850,12 @@
       <c r="U40" s="3"/>
     </row>
     <row r="41" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="21"/>
-      <c r="B41" s="21"/>
-      <c r="C41" s="21"/>
-      <c r="D41" s="21"/>
-      <c r="E41" s="21"/>
-      <c r="F41" s="21"/>
+      <c r="A41" s="14"/>
+      <c r="B41" s="14"/>
+      <c r="C41" s="14"/>
+      <c r="D41" s="14"/>
+      <c r="E41" s="14"/>
+      <c r="F41" s="14"/>
       <c r="G41" s="3"/>
       <c r="H41" s="3"/>
       <c r="I41" s="3"/>
@@ -4842,12 +4873,12 @@
       <c r="U41" s="3"/>
     </row>
     <row r="42" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="21"/>
-      <c r="B42" s="21"/>
-      <c r="C42" s="21"/>
-      <c r="D42" s="21"/>
-      <c r="E42" s="21"/>
-      <c r="F42" s="21"/>
+      <c r="A42" s="14"/>
+      <c r="B42" s="14"/>
+      <c r="C42" s="14"/>
+      <c r="D42" s="14"/>
+      <c r="E42" s="14"/>
+      <c r="F42" s="14"/>
       <c r="G42" s="3"/>
       <c r="H42" s="3"/>
       <c r="I42" s="3"/>
@@ -6165,13 +6196,13 @@
       <c r="B1" s="6"/>
     </row>
     <row r="2" spans="1:19" ht="37" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="28" t="s">
         <v>139</v>
       </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
     </row>
     <row r="3" spans="1:19" ht="38" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A3" s="12" t="s">
@@ -8196,43 +8227,43 @@
       <c r="B1" s="6"/>
     </row>
     <row r="2" spans="1:19" ht="37" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="28" t="s">
         <v>143</v>
       </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
     </row>
     <row r="3" spans="1:19" ht="38" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="30" t="s">
+      <c r="A3" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="22" t="s">
         <v>144</v>
       </c>
-      <c r="C3" s="31" t="s">
+      <c r="C3" s="23" t="s">
         <v>145</v>
       </c>
-      <c r="D3" s="31" t="s">
+      <c r="D3" s="23" t="s">
         <v>146</v>
       </c>
-      <c r="E3" s="31" t="s">
+      <c r="E3" s="23" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="4" spans="1:19" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="16" t="s">
         <v>187</v>
       </c>
-      <c r="B4" s="23" t="s">
-        <v>233</v>
-      </c>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23" t="s">
+      <c r="B4" s="16" t="s">
+        <v>232</v>
+      </c>
+      <c r="C4" s="16"/>
+      <c r="D4" s="16" t="s">
         <v>188</v>
       </c>
-      <c r="E4" s="23"/>
+      <c r="E4" s="16"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
@@ -8249,18 +8280,18 @@
       <c r="S4" s="2"/>
     </row>
     <row r="5" spans="1:19" ht="118" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="32" t="s">
-        <v>191</v>
-      </c>
-      <c r="B5" s="24" t="s">
-        <v>232</v>
-      </c>
-      <c r="C5" s="33"/>
-      <c r="D5" s="23" t="s">
+      <c r="A5" s="24" t="s">
+        <v>190</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>231</v>
+      </c>
+      <c r="C5" s="25"/>
+      <c r="D5" s="16" t="s">
         <v>188</v>
       </c>
-      <c r="E5" s="23" t="s">
-        <v>216</v>
+      <c r="E5" s="16" t="s">
+        <v>215</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
@@ -8278,11 +8309,19 @@
       <c r="S5" s="2"/>
     </row>
     <row r="6" spans="1:19" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="7"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
+      <c r="A6" s="24" t="s">
+        <v>240</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>241</v>
+      </c>
+      <c r="C6" s="25"/>
+      <c r="D6" s="16" t="s">
+        <v>188</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>242</v>
+      </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>

</xml_diff>

<commit_message>
slow but steady progress, finished categorization, except for Benin
</commit_message>
<xml_diff>
--- a/data/Data Dictionary.xlsx
+++ b/data/Data Dictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stepheaneff/Documents/work/costed-NAPHS/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BA4482F-BD35-ED4D-8B9E-1370386791DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE771B9D-7271-1442-9949-A5433EBE676B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="100" yWindow="760" windowWidth="29780" windowHeight="16820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7480" yWindow="760" windowWidth="29780" windowHeight="16820" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table information" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="261">
   <si>
     <t>Text</t>
   </si>
@@ -769,9 +769,6 @@
     <t>Liberia Costed NAPHS</t>
   </si>
   <si>
-    <t>The data dictionary was last updated on 24 April, 2025</t>
-  </si>
-  <si>
     <t>Requirement highlights</t>
   </si>
   <si>
@@ -782,6 +779,48 @@
   </si>
   <si>
     <t>Generated by research team</t>
+  </si>
+  <si>
+    <t>line_item_id</t>
+  </si>
+  <si>
+    <t>Unique ID</t>
+  </si>
+  <si>
+    <t>A unique line-item ID for each country, requirement, activity, and year</t>
+  </si>
+  <si>
+    <t>manually created by research team (SE) during data cleaning</t>
+  </si>
+  <si>
+    <t>Tagged line items</t>
+  </si>
+  <si>
+    <t>25 April, 2025</t>
+  </si>
+  <si>
+    <t>Added unique IDs to each line item in clean dataset, created separate dataset for the purpose of tagging line-items</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Line Items</t>
+  </si>
+  <si>
+    <t>ICT (included in written description)</t>
+  </si>
+  <si>
+    <t>ICT (Information and Communication Technology)</t>
+  </si>
+  <si>
+    <t>30 April, 2025</t>
+  </si>
+  <si>
+    <t>Added some additional definitions</t>
+  </si>
+  <si>
+    <t>The data dictionary was last updated on 30 April, 2025</t>
   </si>
 </sst>
 </file>
@@ -926,7 +965,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1028,9 +1067,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1045,6 +1081,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1061,23 +1103,17 @@
     <xf numFmtId="0" fontId="12" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="6" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1102,6 +1138,9 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1342,42 +1381,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="29"/>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
+      <c r="A1" s="28"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
     </row>
     <row r="2" spans="1:22" ht="23" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="32" t="s">
+      <c r="A2" s="31" t="s">
         <v>147</v>
       </c>
-      <c r="B2" s="33"/>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
     </row>
     <row r="3" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="30" t="s">
+      <c r="A3" s="29" t="s">
         <v>148</v>
       </c>
-      <c r="B3" s="31"/>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
+      <c r="B3" s="30"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
     </row>
     <row r="4" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="31" t="s">
-        <v>243</v>
-      </c>
-      <c r="B4" s="31"/>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
+      <c r="A4" s="30" t="s">
+        <v>260</v>
+      </c>
+      <c r="B4" s="30"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
     </row>
     <row r="5" spans="1:22" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="31" t="s">
+      <c r="A5" s="30" t="s">
         <v>149</v>
       </c>
-      <c r="B5" s="31"/>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31"/>
+      <c r="B5" s="30"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
     </row>
     <row r="6" spans="1:22" ht="17" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6"/>
@@ -1386,54 +1425,54 @@
       <c r="D6" s="6"/>
     </row>
     <row r="7" spans="1:22" ht="37" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A7" s="28" t="s">
+      <c r="A7" s="27" t="s">
         <v>132</v>
       </c>
-      <c r="B7" s="28"/>
-      <c r="C7" s="28"/>
-      <c r="D7" s="28"/>
-      <c r="E7" s="28"/>
+      <c r="B7" s="27"/>
+      <c r="C7" s="27"/>
+      <c r="D7" s="27"/>
+      <c r="E7" s="27"/>
     </row>
     <row r="8" spans="1:22" ht="32.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="12" t="s">
         <v>152</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="12" t="s">
         <v>134</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="12" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="9" spans="1:22" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="26" t="s">
+      <c r="A9" s="25" t="s">
         <v>192</v>
       </c>
-      <c r="B9" s="26"/>
-      <c r="C9" s="26"/>
-      <c r="D9" s="26"/>
-      <c r="E9" s="26"/>
+      <c r="B9" s="25"/>
+      <c r="C9" s="25"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="25"/>
     </row>
     <row r="10" spans="1:22" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="15" t="s">
+      <c r="A10" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="B10" s="15" t="s">
+      <c r="B10" s="16" t="s">
         <v>154</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="16" t="s">
         <v>153</v>
       </c>
-      <c r="D10" s="15" t="s">
+      <c r="D10" s="16" t="s">
         <v>151</v>
       </c>
-      <c r="E10" s="15" t="s">
+      <c r="E10" s="16" t="s">
         <v>155</v>
       </c>
       <c r="F10" s="2"/>
@@ -1455,13 +1494,13 @@
       <c r="V10" s="2"/>
     </row>
     <row r="11" spans="1:22" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="27" t="s">
+      <c r="A11" s="26" t="s">
         <v>193</v>
       </c>
-      <c r="B11" s="27"/>
-      <c r="C11" s="27"/>
-      <c r="D11" s="27"/>
-      <c r="E11" s="27"/>
+      <c r="B11" s="26"/>
+      <c r="C11" s="26"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="26"/>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
@@ -1481,19 +1520,19 @@
       <c r="V11" s="2"/>
     </row>
     <row r="12" spans="1:22" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="16" t="s">
         <v>189</v>
       </c>
-      <c r="B12" s="15" t="s">
+      <c r="B12" s="16" t="s">
         <v>191</v>
       </c>
-      <c r="C12" s="15" t="s">
+      <c r="C12" s="16" t="s">
         <v>153</v>
       </c>
-      <c r="D12" s="15" t="s">
+      <c r="D12" s="16" t="s">
         <v>151</v>
       </c>
-      <c r="E12" s="15" t="s">
+      <c r="E12" s="16" t="s">
         <v>155</v>
       </c>
       <c r="F12" s="2"/>
@@ -1515,19 +1554,19 @@
       <c r="V12" s="2"/>
     </row>
     <row r="13" spans="1:22" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="16" t="s">
+      <c r="A13" s="17" t="s">
         <v>196</v>
       </c>
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="18" t="s">
         <v>210</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="C13" s="17" t="s">
         <v>211</v>
       </c>
-      <c r="D13" s="16" t="s">
+      <c r="D13" s="17" t="s">
         <v>151</v>
       </c>
-      <c r="E13" s="15" t="s">
+      <c r="E13" s="16" t="s">
         <v>155</v>
       </c>
       <c r="F13" s="2"/>
@@ -1549,19 +1588,19 @@
       <c r="V13" s="2"/>
     </row>
     <row r="14" spans="1:22" ht="97" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="15" t="s">
+      <c r="A14" s="16" t="s">
         <v>212</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="19" t="s">
         <v>213</v>
       </c>
-      <c r="C14" s="15" t="s">
+      <c r="C14" s="16" t="s">
         <v>214</v>
       </c>
-      <c r="D14" s="15" t="s">
+      <c r="D14" s="16" t="s">
         <v>151</v>
       </c>
-      <c r="E14" s="15" t="s">
+      <c r="E14" s="16" t="s">
         <v>215</v>
       </c>
       <c r="F14" s="2"/>
@@ -1583,20 +1622,20 @@
       <c r="V14" s="2"/>
     </row>
     <row r="15" spans="1:22" ht="63" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="16" t="s">
+        <v>243</v>
+      </c>
+      <c r="B15" s="19" t="s">
         <v>244</v>
       </c>
-      <c r="B15" s="18" t="s">
+      <c r="C15" s="16" t="s">
         <v>245</v>
       </c>
-      <c r="C15" s="15" t="s">
+      <c r="D15" s="16" t="s">
+        <v>151</v>
+      </c>
+      <c r="E15" s="16" t="s">
         <v>246</v>
-      </c>
-      <c r="D15" s="15" t="s">
-        <v>151</v>
-      </c>
-      <c r="E15" s="15" t="s">
-        <v>247</v>
       </c>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
@@ -1616,12 +1655,22 @@
       <c r="U15" s="2"/>
       <c r="V15" s="2"/>
     </row>
-    <row r="16" spans="1:22" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="7"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="2"/>
+    <row r="16" spans="1:22" ht="63" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="16" t="s">
+        <v>251</v>
+      </c>
+      <c r="B16" s="19" t="s">
+        <v>244</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>245</v>
+      </c>
+      <c r="D16" s="16" t="s">
+        <v>151</v>
+      </c>
+      <c r="E16" s="16" t="s">
+        <v>246</v>
+      </c>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
@@ -3641,7 +3690,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U1003"/>
+  <dimension ref="A1:U1004"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.3984375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35.19921875" customWidth="1"/>
@@ -3659,98 +3708,83 @@
       <c r="D1" s="6"/>
     </row>
     <row r="2" spans="1:21" ht="37" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="27" t="s">
         <v>136</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
     </row>
     <row r="3" spans="1:21" ht="30" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="12" t="s">
         <v>137</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="F3" s="12" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="4" spans="1:21" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="26" t="s">
+      <c r="A4" s="25" t="s">
         <v>194</v>
       </c>
-      <c r="B4" s="26"/>
-      <c r="C4" s="26"/>
-      <c r="D4" s="26"/>
-      <c r="E4" s="26"/>
-      <c r="F4" s="26"/>
-    </row>
-    <row r="5" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="15" t="s">
+      <c r="B4" s="25"/>
+      <c r="C4" s="25"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="25"/>
+    </row>
+    <row r="5" spans="1:21" ht="46" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="16" t="s">
+        <v>247</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>248</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>249</v>
+      </c>
+      <c r="E5" s="16" t="s">
+        <v>184</v>
+      </c>
+      <c r="F5" s="24" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="16" t="s">
+        <v>150</v>
+      </c>
+      <c r="B6" s="16" t="s">
         <v>174</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C6" s="16" t="s">
         <v>156</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="D6" s="16" t="s">
         <v>165</v>
       </c>
-      <c r="E5" s="15" t="s">
+      <c r="E6" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="F5" s="15" t="s">
+      <c r="F6" s="16" t="s">
         <v>186</v>
-      </c>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2"/>
-      <c r="M5" s="2"/>
-      <c r="N5" s="2"/>
-      <c r="O5" s="2"/>
-      <c r="P5" s="2"/>
-      <c r="Q5" s="2"/>
-      <c r="R5" s="2"/>
-      <c r="S5" s="2"/>
-      <c r="T5" s="2"/>
-      <c r="U5" s="2"/>
-    </row>
-    <row r="6" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="15" t="s">
-        <v>150</v>
-      </c>
-      <c r="B6" s="15" t="s">
-        <v>197</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>198</v>
-      </c>
-      <c r="D6" s="19" t="s">
-        <v>208</v>
-      </c>
-      <c r="E6" s="15" t="s">
-        <v>183</v>
-      </c>
-      <c r="F6" s="20" t="s">
-        <v>209</v>
       </c>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
@@ -3769,23 +3803,23 @@
       <c r="U6" s="2"/>
     </row>
     <row r="7" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="B7" s="18" t="s">
-        <v>175</v>
-      </c>
-      <c r="C7" s="18" t="s">
-        <v>157</v>
-      </c>
-      <c r="D7" s="19" t="s">
-        <v>207</v>
-      </c>
-      <c r="E7" s="15" t="s">
+      <c r="B7" s="16" t="s">
+        <v>197</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>198</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>208</v>
+      </c>
+      <c r="E7" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="F7" s="15" t="s">
-        <v>186</v>
+      <c r="F7" s="24" t="s">
+        <v>209</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
@@ -3804,22 +3838,22 @@
       <c r="U7" s="2"/>
     </row>
     <row r="8" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="15" t="s">
+      <c r="A8" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="B8" s="18" t="s">
-        <v>176</v>
-      </c>
-      <c r="C8" s="15" t="s">
-        <v>158</v>
-      </c>
-      <c r="D8" s="19" t="s">
-        <v>167</v>
-      </c>
-      <c r="E8" s="15" t="s">
+      <c r="B8" s="19" t="s">
+        <v>175</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>157</v>
+      </c>
+      <c r="D8" s="20" t="s">
+        <v>207</v>
+      </c>
+      <c r="E8" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="F8" s="15" t="s">
+      <c r="F8" s="16" t="s">
         <v>186</v>
       </c>
       <c r="G8" s="2"/>
@@ -3839,22 +3873,22 @@
       <c r="U8" s="2"/>
     </row>
     <row r="9" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="B9" s="18" t="s">
-        <v>177</v>
-      </c>
-      <c r="C9" s="15" t="s">
-        <v>159</v>
-      </c>
-      <c r="D9" s="19" t="s">
-        <v>168</v>
-      </c>
-      <c r="E9" s="15" t="s">
+      <c r="B9" s="19" t="s">
+        <v>176</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>158</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>167</v>
+      </c>
+      <c r="E9" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="F9" s="15" t="s">
+      <c r="F9" s="16" t="s">
         <v>186</v>
       </c>
       <c r="G9" s="2"/>
@@ -3874,22 +3908,22 @@
       <c r="U9" s="2"/>
     </row>
     <row r="10" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="15" t="s">
+      <c r="A10" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="B10" s="18" t="s">
-        <v>178</v>
-      </c>
-      <c r="C10" s="15" t="s">
-        <v>160</v>
-      </c>
-      <c r="D10" s="15" t="s">
-        <v>169</v>
-      </c>
-      <c r="E10" s="15" t="s">
-        <v>184</v>
-      </c>
-      <c r="F10" s="15" t="s">
+      <c r="B10" s="19" t="s">
+        <v>177</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>159</v>
+      </c>
+      <c r="D10" s="20" t="s">
+        <v>168</v>
+      </c>
+      <c r="E10" s="16" t="s">
+        <v>183</v>
+      </c>
+      <c r="F10" s="16" t="s">
         <v>186</v>
       </c>
       <c r="G10" s="2"/>
@@ -3909,22 +3943,22 @@
       <c r="U10" s="2"/>
     </row>
     <row r="11" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="B11" s="18" t="s">
-        <v>179</v>
-      </c>
-      <c r="C11" s="18" t="s">
-        <v>161</v>
-      </c>
-      <c r="D11" s="15" t="s">
-        <v>170</v>
-      </c>
-      <c r="E11" s="15" t="s">
+      <c r="B11" s="19" t="s">
+        <v>178</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>160</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>169</v>
+      </c>
+      <c r="E11" s="16" t="s">
         <v>184</v>
       </c>
-      <c r="F11" s="15" t="s">
+      <c r="F11" s="16" t="s">
         <v>186</v>
       </c>
       <c r="G11" s="2"/>
@@ -3944,22 +3978,22 @@
       <c r="U11" s="2"/>
     </row>
     <row r="12" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="B12" s="18" t="s">
-        <v>233</v>
-      </c>
-      <c r="C12" s="18" t="s">
-        <v>234</v>
-      </c>
-      <c r="D12" s="15" t="s">
-        <v>235</v>
-      </c>
-      <c r="E12" s="15" t="s">
-        <v>185</v>
-      </c>
-      <c r="F12" s="15" t="s">
+      <c r="B12" s="19" t="s">
+        <v>179</v>
+      </c>
+      <c r="C12" s="19" t="s">
+        <v>161</v>
+      </c>
+      <c r="D12" s="16" t="s">
+        <v>170</v>
+      </c>
+      <c r="E12" s="16" t="s">
+        <v>184</v>
+      </c>
+      <c r="F12" s="16" t="s">
         <v>186</v>
       </c>
       <c r="G12" s="2"/>
@@ -3979,22 +4013,22 @@
       <c r="U12" s="2"/>
     </row>
     <row r="13" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="15" t="s">
+      <c r="A13" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="B13" s="18" t="s">
-        <v>216</v>
-      </c>
-      <c r="C13" s="18" t="s">
-        <v>221</v>
-      </c>
-      <c r="D13" s="15" t="s">
-        <v>236</v>
-      </c>
-      <c r="E13" s="15" t="s">
-        <v>183</v>
-      </c>
-      <c r="F13" s="15" t="s">
+      <c r="B13" s="19" t="s">
+        <v>233</v>
+      </c>
+      <c r="C13" s="19" t="s">
+        <v>234</v>
+      </c>
+      <c r="D13" s="16" t="s">
+        <v>235</v>
+      </c>
+      <c r="E13" s="16" t="s">
+        <v>185</v>
+      </c>
+      <c r="F13" s="16" t="s">
         <v>186</v>
       </c>
       <c r="G13" s="2"/>
@@ -4013,24 +4047,24 @@
       <c r="T13" s="2"/>
       <c r="U13" s="2"/>
     </row>
-    <row r="14" spans="1:21" ht="84" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="15" t="s">
+    <row r="14" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="B14" s="18" t="s">
-        <v>237</v>
-      </c>
-      <c r="C14" s="18" t="s">
-        <v>238</v>
-      </c>
-      <c r="D14" s="15" t="s">
-        <v>239</v>
-      </c>
-      <c r="E14" s="15" t="s">
-        <v>185</v>
-      </c>
-      <c r="F14" s="15" t="s">
-        <v>215</v>
+      <c r="B14" s="19" t="s">
+        <v>216</v>
+      </c>
+      <c r="C14" s="19" t="s">
+        <v>221</v>
+      </c>
+      <c r="D14" s="16" t="s">
+        <v>236</v>
+      </c>
+      <c r="E14" s="16" t="s">
+        <v>183</v>
+      </c>
+      <c r="F14" s="16" t="s">
+        <v>186</v>
       </c>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
@@ -4048,24 +4082,24 @@
       <c r="T14" s="2"/>
       <c r="U14" s="2"/>
     </row>
-    <row r="15" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="15" t="s">
+    <row r="15" spans="1:21" ht="84" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="B15" s="15" t="s">
-        <v>182</v>
-      </c>
-      <c r="C15" s="18" t="s">
-        <v>164</v>
-      </c>
-      <c r="D15" s="15" t="s">
-        <v>173</v>
-      </c>
-      <c r="E15" s="15" t="s">
-        <v>183</v>
-      </c>
-      <c r="F15" s="15" t="s">
-        <v>186</v>
+      <c r="B15" s="19" t="s">
+        <v>237</v>
+      </c>
+      <c r="C15" s="19" t="s">
+        <v>238</v>
+      </c>
+      <c r="D15" s="16" t="s">
+        <v>239</v>
+      </c>
+      <c r="E15" s="16" t="s">
+        <v>185</v>
+      </c>
+      <c r="F15" s="16" t="s">
+        <v>215</v>
       </c>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
@@ -4083,68 +4117,68 @@
       <c r="T15" s="2"/>
       <c r="U15" s="2"/>
     </row>
-    <row r="16" spans="1:21" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="27" t="s">
+    <row r="16" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="16" t="s">
+        <v>150</v>
+      </c>
+      <c r="B16" s="16" t="s">
+        <v>182</v>
+      </c>
+      <c r="C16" s="19" t="s">
+        <v>164</v>
+      </c>
+      <c r="D16" s="16" t="s">
+        <v>173</v>
+      </c>
+      <c r="E16" s="16" t="s">
+        <v>183</v>
+      </c>
+      <c r="F16" s="16" t="s">
+        <v>186</v>
+      </c>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
+      <c r="L16" s="2"/>
+      <c r="M16" s="2"/>
+      <c r="N16" s="2"/>
+      <c r="O16" s="2"/>
+      <c r="P16" s="2"/>
+      <c r="Q16" s="2"/>
+      <c r="R16" s="2"/>
+      <c r="S16" s="2"/>
+      <c r="T16" s="2"/>
+      <c r="U16" s="2"/>
+    </row>
+    <row r="17" spans="1:21" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="26" t="s">
         <v>195</v>
       </c>
-      <c r="B16" s="27"/>
-      <c r="C16" s="27"/>
-      <c r="D16" s="27"/>
-      <c r="E16" s="27"/>
-      <c r="F16" s="27"/>
-    </row>
-    <row r="17" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="15" t="s">
+      <c r="B17" s="26"/>
+      <c r="C17" s="26"/>
+      <c r="D17" s="26"/>
+      <c r="E17" s="26"/>
+      <c r="F17" s="26"/>
+    </row>
+    <row r="18" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="16" t="s">
         <v>189</v>
       </c>
-      <c r="B17" s="15" t="s">
+      <c r="B18" s="16" t="s">
         <v>174</v>
       </c>
-      <c r="C17" s="15" t="s">
+      <c r="C18" s="16" t="s">
         <v>156</v>
       </c>
-      <c r="D17" s="15" t="s">
+      <c r="D18" s="16" t="s">
         <v>165</v>
       </c>
-      <c r="E17" s="15" t="s">
+      <c r="E18" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="F17" s="15" t="s">
-        <v>186</v>
-      </c>
-      <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
-      <c r="L17" s="2"/>
-      <c r="M17" s="2"/>
-      <c r="N17" s="2"/>
-      <c r="O17" s="2"/>
-      <c r="P17" s="2"/>
-      <c r="Q17" s="2"/>
-      <c r="R17" s="2"/>
-      <c r="S17" s="2"/>
-      <c r="T17" s="2"/>
-      <c r="U17" s="2"/>
-    </row>
-    <row r="18" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="15" t="s">
-        <v>189</v>
-      </c>
-      <c r="B18" s="18" t="s">
-        <v>175</v>
-      </c>
-      <c r="C18" s="18" t="s">
-        <v>157</v>
-      </c>
-      <c r="D18" s="19" t="s">
-        <v>166</v>
-      </c>
-      <c r="E18" s="15" t="s">
-        <v>183</v>
-      </c>
-      <c r="F18" s="15" t="s">
+      <c r="F18" s="16" t="s">
         <v>186</v>
       </c>
       <c r="G18" s="2"/>
@@ -4164,22 +4198,22 @@
       <c r="U18" s="2"/>
     </row>
     <row r="19" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="15" t="s">
+      <c r="A19" s="16" t="s">
         <v>189</v>
       </c>
-      <c r="B19" s="18" t="s">
-        <v>176</v>
-      </c>
-      <c r="C19" s="15" t="s">
-        <v>158</v>
-      </c>
-      <c r="D19" s="19" t="s">
-        <v>167</v>
-      </c>
-      <c r="E19" s="15" t="s">
+      <c r="B19" s="19" t="s">
+        <v>175</v>
+      </c>
+      <c r="C19" s="19" t="s">
+        <v>157</v>
+      </c>
+      <c r="D19" s="20" t="s">
+        <v>166</v>
+      </c>
+      <c r="E19" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="F19" s="15" t="s">
+      <c r="F19" s="16" t="s">
         <v>186</v>
       </c>
       <c r="G19" s="2"/>
@@ -4199,22 +4233,22 @@
       <c r="U19" s="2"/>
     </row>
     <row r="20" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="15" t="s">
+      <c r="A20" s="16" t="s">
         <v>189</v>
       </c>
-      <c r="B20" s="18" t="s">
-        <v>177</v>
-      </c>
-      <c r="C20" s="15" t="s">
-        <v>159</v>
-      </c>
-      <c r="D20" s="19" t="s">
-        <v>168</v>
-      </c>
-      <c r="E20" s="15" t="s">
+      <c r="B20" s="19" t="s">
+        <v>176</v>
+      </c>
+      <c r="C20" s="16" t="s">
+        <v>158</v>
+      </c>
+      <c r="D20" s="20" t="s">
+        <v>167</v>
+      </c>
+      <c r="E20" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="F20" s="15" t="s">
+      <c r="F20" s="16" t="s">
         <v>186</v>
       </c>
       <c r="G20" s="2"/>
@@ -4234,22 +4268,22 @@
       <c r="U20" s="2"/>
     </row>
     <row r="21" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="15" t="s">
+      <c r="A21" s="16" t="s">
         <v>189</v>
       </c>
-      <c r="B21" s="18" t="s">
-        <v>178</v>
-      </c>
-      <c r="C21" s="15" t="s">
-        <v>160</v>
-      </c>
-      <c r="D21" s="15" t="s">
-        <v>169</v>
-      </c>
-      <c r="E21" s="15" t="s">
-        <v>184</v>
-      </c>
-      <c r="F21" s="15" t="s">
+      <c r="B21" s="19" t="s">
+        <v>177</v>
+      </c>
+      <c r="C21" s="16" t="s">
+        <v>159</v>
+      </c>
+      <c r="D21" s="20" t="s">
+        <v>168</v>
+      </c>
+      <c r="E21" s="16" t="s">
+        <v>183</v>
+      </c>
+      <c r="F21" s="16" t="s">
         <v>186</v>
       </c>
       <c r="G21" s="2"/>
@@ -4269,22 +4303,22 @@
       <c r="U21" s="2"/>
     </row>
     <row r="22" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="15" t="s">
+      <c r="A22" s="16" t="s">
         <v>189</v>
       </c>
-      <c r="B22" s="18" t="s">
-        <v>179</v>
-      </c>
-      <c r="C22" s="18" t="s">
-        <v>161</v>
-      </c>
-      <c r="D22" s="15" t="s">
-        <v>170</v>
-      </c>
-      <c r="E22" s="15" t="s">
+      <c r="B22" s="19" t="s">
+        <v>178</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>160</v>
+      </c>
+      <c r="D22" s="16" t="s">
+        <v>169</v>
+      </c>
+      <c r="E22" s="16" t="s">
         <v>184</v>
       </c>
-      <c r="F22" s="15" t="s">
+      <c r="F22" s="16" t="s">
         <v>186</v>
       </c>
       <c r="G22" s="2"/>
@@ -4304,22 +4338,22 @@
       <c r="U22" s="2"/>
     </row>
     <row r="23" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="15" t="s">
+      <c r="A23" s="16" t="s">
         <v>189</v>
       </c>
-      <c r="B23" s="18" t="s">
-        <v>180</v>
-      </c>
-      <c r="C23" s="18" t="s">
-        <v>162</v>
-      </c>
-      <c r="D23" s="15" t="s">
-        <v>171</v>
-      </c>
-      <c r="E23" s="15" t="s">
-        <v>185</v>
-      </c>
-      <c r="F23" s="15" t="s">
+      <c r="B23" s="19" t="s">
+        <v>179</v>
+      </c>
+      <c r="C23" s="19" t="s">
+        <v>161</v>
+      </c>
+      <c r="D23" s="16" t="s">
+        <v>170</v>
+      </c>
+      <c r="E23" s="16" t="s">
+        <v>184</v>
+      </c>
+      <c r="F23" s="16" t="s">
         <v>186</v>
       </c>
       <c r="G23" s="2"/>
@@ -4339,22 +4373,22 @@
       <c r="U23" s="2"/>
     </row>
     <row r="24" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="15" t="s">
+      <c r="A24" s="16" t="s">
         <v>189</v>
       </c>
-      <c r="B24" s="18" t="s">
-        <v>181</v>
-      </c>
-      <c r="C24" s="18" t="s">
-        <v>163</v>
-      </c>
-      <c r="D24" s="15" t="s">
-        <v>172</v>
-      </c>
-      <c r="E24" s="15" t="s">
-        <v>183</v>
-      </c>
-      <c r="F24" s="15" t="s">
+      <c r="B24" s="19" t="s">
+        <v>180</v>
+      </c>
+      <c r="C24" s="19" t="s">
+        <v>162</v>
+      </c>
+      <c r="D24" s="16" t="s">
+        <v>171</v>
+      </c>
+      <c r="E24" s="16" t="s">
+        <v>185</v>
+      </c>
+      <c r="F24" s="16" t="s">
         <v>186</v>
       </c>
       <c r="G24" s="2"/>
@@ -4374,22 +4408,22 @@
       <c r="U24" s="2"/>
     </row>
     <row r="25" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="15" t="s">
+      <c r="A25" s="16" t="s">
         <v>189</v>
       </c>
-      <c r="B25" s="15" t="s">
-        <v>182</v>
-      </c>
-      <c r="C25" s="18" t="s">
-        <v>164</v>
-      </c>
-      <c r="D25" s="15" t="s">
-        <v>173</v>
-      </c>
-      <c r="E25" s="15" t="s">
+      <c r="B25" s="19" t="s">
+        <v>181</v>
+      </c>
+      <c r="C25" s="19" t="s">
+        <v>163</v>
+      </c>
+      <c r="D25" s="16" t="s">
+        <v>172</v>
+      </c>
+      <c r="E25" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="F25" s="15" t="s">
+      <c r="F25" s="16" t="s">
         <v>186</v>
       </c>
       <c r="G25" s="2"/>
@@ -4409,23 +4443,23 @@
       <c r="U25" s="2"/>
     </row>
     <row r="26" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="15" t="s">
-        <v>196</v>
-      </c>
-      <c r="B26" s="15" t="s">
-        <v>197</v>
-      </c>
-      <c r="C26" s="15" t="s">
-        <v>198</v>
-      </c>
-      <c r="D26" s="21" t="s">
-        <v>203</v>
-      </c>
-      <c r="E26" s="15" t="s">
+      <c r="A26" s="16" t="s">
+        <v>189</v>
+      </c>
+      <c r="B26" s="16" t="s">
+        <v>182</v>
+      </c>
+      <c r="C26" s="19" t="s">
+        <v>164</v>
+      </c>
+      <c r="D26" s="16" t="s">
+        <v>173</v>
+      </c>
+      <c r="E26" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="F26" s="21" t="s">
-        <v>206</v>
+      <c r="F26" s="16" t="s">
+        <v>186</v>
       </c>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
@@ -4444,19 +4478,19 @@
       <c r="U26" s="2"/>
     </row>
     <row r="27" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="15" t="s">
+      <c r="A27" s="16" t="s">
         <v>196</v>
       </c>
-      <c r="B27" s="15" t="s">
-        <v>199</v>
-      </c>
-      <c r="C27" s="15" t="s">
-        <v>201</v>
+      <c r="B27" s="16" t="s">
+        <v>197</v>
+      </c>
+      <c r="C27" s="16" t="s">
+        <v>198</v>
       </c>
       <c r="D27" s="21" t="s">
-        <v>204</v>
-      </c>
-      <c r="E27" s="15" t="s">
+        <v>203</v>
+      </c>
+      <c r="E27" s="16" t="s">
         <v>183</v>
       </c>
       <c r="F27" s="21" t="s">
@@ -4479,19 +4513,19 @@
       <c r="U27" s="2"/>
     </row>
     <row r="28" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="15" t="s">
+      <c r="A28" s="16" t="s">
         <v>196</v>
       </c>
-      <c r="B28" s="15" t="s">
-        <v>200</v>
-      </c>
-      <c r="C28" s="15" t="s">
-        <v>202</v>
+      <c r="B28" s="16" t="s">
+        <v>199</v>
+      </c>
+      <c r="C28" s="16" t="s">
+        <v>201</v>
       </c>
       <c r="D28" s="21" t="s">
-        <v>205</v>
-      </c>
-      <c r="E28" s="15" t="s">
+        <v>204</v>
+      </c>
+      <c r="E28" s="16" t="s">
         <v>183</v>
       </c>
       <c r="F28" s="21" t="s">
@@ -4513,24 +4547,24 @@
       <c r="T28" s="2"/>
       <c r="U28" s="2"/>
     </row>
-    <row r="29" spans="1:21" ht="84" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="15" t="s">
-        <v>212</v>
-      </c>
-      <c r="B29" s="15" t="s">
-        <v>216</v>
-      </c>
-      <c r="C29" s="15" t="s">
-        <v>221</v>
+    <row r="29" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="16" t="s">
+        <v>196</v>
+      </c>
+      <c r="B29" s="16" t="s">
+        <v>200</v>
+      </c>
+      <c r="C29" s="16" t="s">
+        <v>202</v>
       </c>
       <c r="D29" s="21" t="s">
-        <v>226</v>
-      </c>
-      <c r="E29" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="E29" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="F29" s="15" t="s">
-        <v>215</v>
+      <c r="F29" s="21" t="s">
+        <v>206</v>
       </c>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
@@ -4548,23 +4582,23 @@
       <c r="T29" s="2"/>
       <c r="U29" s="2"/>
     </row>
-    <row r="30" spans="1:21" ht="82" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="15" t="s">
+    <row r="30" spans="1:21" ht="84" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="16" t="s">
         <v>212</v>
       </c>
-      <c r="B30" s="15" t="s">
-        <v>217</v>
-      </c>
-      <c r="C30" s="15" t="s">
-        <v>222</v>
-      </c>
-      <c r="D30" s="15" t="s">
-        <v>227</v>
-      </c>
-      <c r="E30" s="15" t="s">
+      <c r="B30" s="16" t="s">
+        <v>216</v>
+      </c>
+      <c r="C30" s="16" t="s">
+        <v>221</v>
+      </c>
+      <c r="D30" s="21" t="s">
+        <v>226</v>
+      </c>
+      <c r="E30" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="F30" s="15" t="s">
+      <c r="F30" s="16" t="s">
         <v>215</v>
       </c>
       <c r="G30" s="2"/>
@@ -4584,22 +4618,22 @@
       <c r="U30" s="2"/>
     </row>
     <row r="31" spans="1:21" ht="82" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="15" t="s">
+      <c r="A31" s="16" t="s">
         <v>212</v>
       </c>
-      <c r="B31" s="15" t="s">
-        <v>218</v>
-      </c>
-      <c r="C31" s="15" t="s">
-        <v>223</v>
-      </c>
-      <c r="D31" s="15" t="s">
-        <v>228</v>
-      </c>
-      <c r="E31" s="15" t="s">
-        <v>185</v>
-      </c>
-      <c r="F31" s="15" t="s">
+      <c r="B31" s="16" t="s">
+        <v>217</v>
+      </c>
+      <c r="C31" s="16" t="s">
+        <v>222</v>
+      </c>
+      <c r="D31" s="16" t="s">
+        <v>227</v>
+      </c>
+      <c r="E31" s="16" t="s">
+        <v>183</v>
+      </c>
+      <c r="F31" s="16" t="s">
         <v>215</v>
       </c>
       <c r="G31" s="2"/>
@@ -4618,23 +4652,23 @@
       <c r="T31" s="2"/>
       <c r="U31" s="2"/>
     </row>
-    <row r="32" spans="1:21" ht="83" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="15" t="s">
+    <row r="32" spans="1:21" ht="82" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="16" t="s">
         <v>212</v>
       </c>
-      <c r="B32" s="15" t="s">
-        <v>219</v>
-      </c>
-      <c r="C32" s="15" t="s">
-        <v>224</v>
-      </c>
-      <c r="D32" s="15" t="s">
-        <v>229</v>
-      </c>
-      <c r="E32" s="15" t="s">
-        <v>183</v>
-      </c>
-      <c r="F32" s="15" t="s">
+      <c r="B32" s="16" t="s">
+        <v>218</v>
+      </c>
+      <c r="C32" s="16" t="s">
+        <v>223</v>
+      </c>
+      <c r="D32" s="16" t="s">
+        <v>228</v>
+      </c>
+      <c r="E32" s="16" t="s">
+        <v>185</v>
+      </c>
+      <c r="F32" s="16" t="s">
         <v>215</v>
       </c>
       <c r="G32" s="2"/>
@@ -4654,22 +4688,22 @@
       <c r="U32" s="2"/>
     </row>
     <row r="33" spans="1:21" ht="83" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="15" t="s">
+      <c r="A33" s="16" t="s">
         <v>212</v>
       </c>
-      <c r="B33" s="15" t="s">
-        <v>220</v>
-      </c>
-      <c r="C33" s="15" t="s">
-        <v>225</v>
-      </c>
-      <c r="D33" s="15" t="s">
-        <v>230</v>
-      </c>
-      <c r="E33" s="15" t="s">
+      <c r="B33" s="16" t="s">
+        <v>219</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>224</v>
+      </c>
+      <c r="D33" s="16" t="s">
+        <v>229</v>
+      </c>
+      <c r="E33" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="F33" s="15" t="s">
+      <c r="F33" s="16" t="s">
         <v>215</v>
       </c>
       <c r="G33" s="2"/>
@@ -4688,13 +4722,25 @@
       <c r="T33" s="2"/>
       <c r="U33" s="2"/>
     </row>
-    <row r="34" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="11"/>
-      <c r="B34" s="11"/>
-      <c r="C34" s="11"/>
-      <c r="D34" s="11"/>
-      <c r="E34" s="14"/>
-      <c r="F34" s="14"/>
+    <row r="34" spans="1:21" ht="83" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="16" t="s">
+        <v>212</v>
+      </c>
+      <c r="B34" s="16" t="s">
+        <v>220</v>
+      </c>
+      <c r="C34" s="16" t="s">
+        <v>225</v>
+      </c>
+      <c r="D34" s="16" t="s">
+        <v>230</v>
+      </c>
+      <c r="E34" s="16" t="s">
+        <v>183</v>
+      </c>
+      <c r="F34" s="16" t="s">
+        <v>215</v>
+      </c>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
       <c r="I34" s="2"/>
@@ -4712,12 +4758,12 @@
       <c r="U34" s="2"/>
     </row>
     <row r="35" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="11"/>
-      <c r="B35" s="11"/>
-      <c r="C35" s="11"/>
-      <c r="D35" s="11"/>
-      <c r="E35" s="14"/>
-      <c r="F35" s="14"/>
+      <c r="A35" s="10"/>
+      <c r="B35" s="10"/>
+      <c r="C35" s="10"/>
+      <c r="D35" s="10"/>
+      <c r="E35" s="13"/>
+      <c r="F35" s="13"/>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="2"/>
@@ -4735,35 +4781,35 @@
       <c r="U35" s="2"/>
     </row>
     <row r="36" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="11"/>
-      <c r="B36" s="11"/>
-      <c r="C36" s="11"/>
-      <c r="D36" s="11"/>
-      <c r="E36" s="14"/>
-      <c r="F36" s="14"/>
-      <c r="G36" s="3"/>
-      <c r="H36" s="3"/>
-      <c r="I36" s="3"/>
-      <c r="J36" s="3"/>
-      <c r="K36" s="3"/>
-      <c r="L36" s="3"/>
-      <c r="M36" s="3"/>
-      <c r="N36" s="3"/>
-      <c r="O36" s="3"/>
-      <c r="P36" s="3"/>
-      <c r="Q36" s="3"/>
-      <c r="R36" s="3"/>
-      <c r="S36" s="3"/>
-      <c r="T36" s="3"/>
-      <c r="U36" s="3"/>
+      <c r="A36" s="10"/>
+      <c r="B36" s="10"/>
+      <c r="C36" s="10"/>
+      <c r="D36" s="10"/>
+      <c r="E36" s="13"/>
+      <c r="F36" s="13"/>
+      <c r="G36" s="2"/>
+      <c r="H36" s="2"/>
+      <c r="I36" s="2"/>
+      <c r="J36" s="2"/>
+      <c r="K36" s="2"/>
+      <c r="L36" s="2"/>
+      <c r="M36" s="2"/>
+      <c r="N36" s="2"/>
+      <c r="O36" s="2"/>
+      <c r="P36" s="2"/>
+      <c r="Q36" s="2"/>
+      <c r="R36" s="2"/>
+      <c r="S36" s="2"/>
+      <c r="T36" s="2"/>
+      <c r="U36" s="2"/>
     </row>
     <row r="37" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="11"/>
-      <c r="B37" s="11"/>
-      <c r="C37" s="11"/>
-      <c r="D37" s="11"/>
-      <c r="E37" s="14"/>
-      <c r="F37" s="14"/>
+      <c r="A37" s="10"/>
+      <c r="B37" s="10"/>
+      <c r="C37" s="10"/>
+      <c r="D37" s="10"/>
+      <c r="E37" s="13"/>
+      <c r="F37" s="13"/>
       <c r="G37" s="3"/>
       <c r="H37" s="3"/>
       <c r="I37" s="3"/>
@@ -4781,12 +4827,12 @@
       <c r="U37" s="3"/>
     </row>
     <row r="38" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="11"/>
-      <c r="B38" s="11"/>
-      <c r="C38" s="11"/>
-      <c r="D38" s="11"/>
-      <c r="E38" s="14"/>
-      <c r="F38" s="14"/>
+      <c r="A38" s="10"/>
+      <c r="B38" s="10"/>
+      <c r="C38" s="10"/>
+      <c r="D38" s="10"/>
+      <c r="E38" s="13"/>
+      <c r="F38" s="13"/>
       <c r="G38" s="3"/>
       <c r="H38" s="3"/>
       <c r="I38" s="3"/>
@@ -4804,12 +4850,12 @@
       <c r="U38" s="3"/>
     </row>
     <row r="39" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="11"/>
-      <c r="B39" s="11"/>
-      <c r="C39" s="11"/>
-      <c r="D39" s="11"/>
-      <c r="E39" s="14"/>
-      <c r="F39" s="14"/>
+      <c r="A39" s="10"/>
+      <c r="B39" s="10"/>
+      <c r="C39" s="10"/>
+      <c r="D39" s="10"/>
+      <c r="E39" s="13"/>
+      <c r="F39" s="13"/>
       <c r="G39" s="3"/>
       <c r="H39" s="3"/>
       <c r="I39" s="3"/>
@@ -4827,12 +4873,12 @@
       <c r="U39" s="3"/>
     </row>
     <row r="40" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="11"/>
-      <c r="B40" s="11"/>
-      <c r="C40" s="11"/>
-      <c r="D40" s="11"/>
-      <c r="E40" s="14"/>
-      <c r="F40" s="14"/>
+      <c r="A40" s="10"/>
+      <c r="B40" s="10"/>
+      <c r="C40" s="10"/>
+      <c r="D40" s="10"/>
+      <c r="E40" s="13"/>
+      <c r="F40" s="13"/>
       <c r="G40" s="3"/>
       <c r="H40" s="3"/>
       <c r="I40" s="3"/>
@@ -4850,12 +4896,12 @@
       <c r="U40" s="3"/>
     </row>
     <row r="41" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="14"/>
-      <c r="B41" s="14"/>
-      <c r="C41" s="14"/>
-      <c r="D41" s="14"/>
-      <c r="E41" s="14"/>
-      <c r="F41" s="14"/>
+      <c r="A41" s="10"/>
+      <c r="B41" s="10"/>
+      <c r="C41" s="10"/>
+      <c r="D41" s="10"/>
+      <c r="E41" s="13"/>
+      <c r="F41" s="13"/>
       <c r="G41" s="3"/>
       <c r="H41" s="3"/>
       <c r="I41" s="3"/>
@@ -4873,12 +4919,12 @@
       <c r="U41" s="3"/>
     </row>
     <row r="42" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="14"/>
-      <c r="B42" s="14"/>
-      <c r="C42" s="14"/>
-      <c r="D42" s="14"/>
-      <c r="E42" s="14"/>
-      <c r="F42" s="14"/>
+      <c r="A42" s="13"/>
+      <c r="B42" s="13"/>
+      <c r="C42" s="13"/>
+      <c r="D42" s="13"/>
+      <c r="E42" s="13"/>
+      <c r="F42" s="13"/>
       <c r="G42" s="3"/>
       <c r="H42" s="3"/>
       <c r="I42" s="3"/>
@@ -4896,12 +4942,12 @@
       <c r="U42" s="3"/>
     </row>
     <row r="43" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="3"/>
-      <c r="B43" s="3"/>
-      <c r="C43" s="3"/>
-      <c r="D43" s="3"/>
-      <c r="E43" s="3"/>
-      <c r="F43" s="3"/>
+      <c r="A43" s="13"/>
+      <c r="B43" s="13"/>
+      <c r="C43" s="13"/>
+      <c r="D43" s="13"/>
+      <c r="E43" s="13"/>
+      <c r="F43" s="13"/>
       <c r="G43" s="3"/>
       <c r="H43" s="3"/>
       <c r="I43" s="3"/>
@@ -5171,7 +5217,7 @@
       <c r="T54" s="3"/>
       <c r="U54" s="3"/>
     </row>
-    <row r="55" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="3"/>
       <c r="B55" s="3"/>
       <c r="C55" s="3"/>
@@ -5217,7 +5263,29 @@
       <c r="T56" s="3"/>
       <c r="U56" s="3"/>
     </row>
-    <row r="57" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="57" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A57" s="3"/>
+      <c r="B57" s="3"/>
+      <c r="C57" s="3"/>
+      <c r="D57" s="3"/>
+      <c r="E57" s="3"/>
+      <c r="F57" s="3"/>
+      <c r="G57" s="3"/>
+      <c r="H57" s="3"/>
+      <c r="I57" s="3"/>
+      <c r="J57" s="3"/>
+      <c r="K57" s="3"/>
+      <c r="L57" s="3"/>
+      <c r="M57" s="3"/>
+      <c r="N57" s="3"/>
+      <c r="O57" s="3"/>
+      <c r="P57" s="3"/>
+      <c r="Q57" s="3"/>
+      <c r="R57" s="3"/>
+      <c r="S57" s="3"/>
+      <c r="T57" s="3"/>
+      <c r="U57" s="3"/>
+    </row>
     <row r="58" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="59" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="60" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -6164,11 +6232,12 @@
     <row r="1001" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="1002" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="1003" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="1004" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A17:F17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape" r:id="rId1"/>
@@ -6186,7 +6255,7 @@
   <cols>
     <col min="1" max="1" width="46" customWidth="1"/>
     <col min="2" max="2" width="36.59765625" customWidth="1"/>
-    <col min="3" max="3" width="38.59765625" customWidth="1"/>
+    <col min="3" max="3" width="46.19921875" customWidth="1"/>
     <col min="4" max="4" width="68.59765625" customWidth="1"/>
     <col min="5" max="5" width="57.59765625" customWidth="1"/>
   </cols>
@@ -6196,38 +6265,46 @@
       <c r="B1" s="6"/>
     </row>
     <row r="2" spans="1:19" ht="37" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="27" t="s">
         <v>139</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
     </row>
     <row r="3" spans="1:19" ht="38" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="12" t="s">
         <v>140</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="12" t="s">
         <v>141</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="12" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="4" spans="1:19" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="10"/>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
+      <c r="A4" s="33" t="s">
+        <v>255</v>
+      </c>
+      <c r="B4" s="33" t="s">
+        <v>159</v>
+      </c>
+      <c r="C4" s="33" t="s">
+        <v>256</v>
+      </c>
+      <c r="D4" s="33" t="s">
+        <v>257</v>
+      </c>
+      <c r="E4" s="33"/>
+      <c r="F4" s="9"/>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
@@ -6243,9 +6320,9 @@
       <c r="S4" s="2"/>
     </row>
     <row r="5" spans="1:19" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="7"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="2"/>
+      <c r="A5" s="33"/>
+      <c r="B5" s="33"/>
+      <c r="C5" s="33"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
@@ -8227,43 +8304,45 @@
       <c r="B1" s="6"/>
     </row>
     <row r="2" spans="1:19" ht="37" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="27" t="s">
         <v>143</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
     </row>
     <row r="3" spans="1:19" ht="38" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="14" t="s">
         <v>144</v>
       </c>
-      <c r="C3" s="23" t="s">
+      <c r="C3" s="15" t="s">
         <v>145</v>
       </c>
-      <c r="D3" s="23" t="s">
+      <c r="D3" s="15" t="s">
         <v>146</v>
       </c>
-      <c r="E3" s="23" t="s">
+      <c r="E3" s="15" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="4" spans="1:19" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="17" t="s">
         <v>232</v>
       </c>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16" t="s">
+      <c r="C4" s="17"/>
+      <c r="D4" s="17" t="s">
         <v>188</v>
       </c>
-      <c r="E4" s="16"/>
+      <c r="E4" s="17" t="s">
+        <v>254</v>
+      </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
@@ -8280,17 +8359,17 @@
       <c r="S4" s="2"/>
     </row>
     <row r="5" spans="1:19" ht="118" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="24" t="s">
+      <c r="A5" s="22" t="s">
         <v>190</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="18" t="s">
         <v>231</v>
       </c>
-      <c r="C5" s="25"/>
-      <c r="D5" s="16" t="s">
+      <c r="C5" s="23"/>
+      <c r="D5" s="17" t="s">
         <v>188</v>
       </c>
-      <c r="E5" s="16" t="s">
+      <c r="E5" s="17" t="s">
         <v>215</v>
       </c>
       <c r="F5" s="2"/>
@@ -8309,17 +8388,17 @@
       <c r="S5" s="2"/>
     </row>
     <row r="6" spans="1:19" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="24" t="s">
+      <c r="A6" s="22" t="s">
         <v>240</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="18" t="s">
         <v>241</v>
       </c>
-      <c r="C6" s="25"/>
-      <c r="D6" s="16" t="s">
+      <c r="C6" s="23"/>
+      <c r="D6" s="17" t="s">
         <v>188</v>
       </c>
-      <c r="E6" s="16" t="s">
+      <c r="E6" s="17" t="s">
         <v>242</v>
       </c>
       <c r="F6" s="2"/>
@@ -8338,11 +8417,19 @@
       <c r="S6" s="2"/>
     </row>
     <row r="7" spans="1:19" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="7"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
+      <c r="A7" s="22" t="s">
+        <v>252</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>253</v>
+      </c>
+      <c r="C7" s="23"/>
+      <c r="D7" s="17" t="s">
+        <v>188</v>
+      </c>
+      <c r="E7" s="17" t="s">
+        <v>254</v>
+      </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
@@ -8359,11 +8446,19 @@
       <c r="S7" s="2"/>
     </row>
     <row r="8" spans="1:19" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="7"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
+      <c r="A8" s="22" t="s">
+        <v>258</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>259</v>
+      </c>
+      <c r="C8" s="23"/>
+      <c r="D8" s="17" t="s">
+        <v>188</v>
+      </c>
+      <c r="E8" s="17" t="s">
+        <v>254</v>
+      </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>

</xml_diff>

<commit_message>
finish summary costs for available countries
</commit_message>
<xml_diff>
--- a/data/Data Dictionary.xlsx
+++ b/data/Data Dictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stepheaneff/Documents/work/GT/costed-NAPHS/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0513CE0C-D7DB-9E4E-89D9-A4D86D9E7806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2FA7F8D-54E8-0947-9341-3B379495179E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="460" yWindow="760" windowWidth="29780" windowHeight="16820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="460" yWindow="760" windowWidth="29780" windowHeight="16820" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="File information" sheetId="2" r:id="rId1"/>
@@ -21,7 +21,7 @@
     <sheet name="Hidden_Agencies" sheetId="6" state="hidden" r:id="rId6"/>
     <sheet name="Hidden_DataTypes" sheetId="7" state="hidden" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="247">
   <si>
     <t>Text</t>
   </si>
@@ -586,12 +586,6 @@
   </si>
   <si>
     <t>The capacity of the JEE to which the cost corresponds, standardized across JEEs (e.g., no numbering or abbreviation)</t>
-  </si>
-  <si>
-    <t>The pillar of the JEE to which the cost corresponds, based on the capacity specified below</t>
-  </si>
-  <si>
-    <t>manually created by research team (SE) based on capacity</t>
   </si>
   <si>
     <t>US Department of Treasury. Fiscal Data, Treasury.gov. Currency Exchange Rates Converter. https://fiscaldata.treasury.gov/currency-exchange-rates-converter/. Accessed 23 April, 2025. 
@@ -676,9 +670,6 @@
     <t>Added some additional definitions</t>
   </si>
   <si>
-    <t>The data dictionary was last updated on 18 November, 2025</t>
-  </si>
-  <si>
     <t>File or dataset</t>
   </si>
   <si>
@@ -769,14 +760,86 @@
     <t>Data extracted from publicly available NAPHS. While Australia completed a publicly available NAPHS, it did not contain any costs (either line-item or summary) and so it is not represented in this dataset.</t>
   </si>
   <si>
-    <t>Afghanistan, Benin, Eritrea</t>
+    <r>
+      <t xml:space="preserve">Afghanistan, Benin, Eritrea,  Liberia, Myanmar, Nigeria, Sierra Leone, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="9" tint="-0.499984740745262"/>
+        <rFont val="Source Sans 3"/>
+      </rPr>
+      <t>South Sudan</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Source Sans 3"/>
+      </rPr>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF014D45"/>
+        <rFont val="Source Sans 3"/>
+      </rPr>
+      <t xml:space="preserve"> Sri Lanka</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Source Sans 3"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF014D45"/>
+        <rFont val="Source Sans 3"/>
+      </rPr>
+      <t>Tanzania</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Source Sans 3"/>
+      </rPr>
+      <t>, Timor-Leste, Uganda</t>
+    </r>
+  </si>
+  <si>
+    <t>The data dictionary was last updated on 29 December, 2025</t>
+  </si>
+  <si>
+    <t>29 December, 2025</t>
+  </si>
+  <si>
+    <t>Added additional summary cost data points ( Liberia, Myanmar, Nigeria, Sierra Leone, South Sudan, Sri Lanka, Tanzania, Timor-Leste, Uganda)</t>
+  </si>
+  <si>
+    <t>The pillar of the JEE to which the cost corresponds, based on the core capacity specified below</t>
+  </si>
+  <si>
+    <t>Pillars defined based on JEE framework</t>
+  </si>
+  <si>
+    <t>US Department of Treasury. Fiscal Data, Treasury.gov. Currency Exchange Rates Converter. https://fiscaldata.treasury.gov/currency-exchange-rates-converter/. Accessed 23 April, 2025. 
+US Bureau of Labor Statistics. CPI Inflation Calculator. https://www.bls.gov/data/inflation_calculator.htm. Accessed 23 April, 2025.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22">
+  <fonts count="24">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -898,6 +961,18 @@
       <b/>
       <sz val="14"/>
       <color rgb="FF000000"/>
+      <name val="Source Sans 3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="9" tint="-0.499984740745262"/>
+      <name val="Source Sans 3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF014D45"/>
       <name val="Source Sans 3"/>
     </font>
   </fonts>
@@ -1101,8 +1176,8 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FF014D45"/>
       <color rgb="FF00A293"/>
-      <color rgb="FF014D45"/>
       <color rgb="FF083F88"/>
       <color rgb="FF009BDF"/>
       <color rgb="FF9C1C28"/>
@@ -1359,7 +1434,7 @@
     </row>
     <row r="4" spans="1:23" ht="22" customHeight="1">
       <c r="A4" s="35" t="s">
-        <v>212</v>
+        <v>241</v>
       </c>
       <c r="B4" s="35"/>
       <c r="C4" s="35"/>
@@ -1384,7 +1459,7 @@
     </row>
     <row r="7" spans="1:23" ht="37" customHeight="1" thickBot="1">
       <c r="A7" s="32" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="B7" s="32"/>
       <c r="C7" s="32"/>
@@ -1394,7 +1469,7 @@
     </row>
     <row r="8" spans="1:23" ht="32.25" customHeight="1" thickTop="1">
       <c r="A8" s="10" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="B8" s="11" t="s">
         <v>2</v>
@@ -1403,7 +1478,7 @@
         <v>150</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="E8" s="11" t="s">
         <v>133</v>
@@ -1414,16 +1489,16 @@
     </row>
     <row r="9" spans="1:23" ht="40" customHeight="1">
       <c r="A9" s="15" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C9" s="15" t="s">
         <v>151</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="E9" s="15" t="s">
         <v>149</v>
@@ -1449,18 +1524,18 @@
       <c r="V9" s="12"/>
       <c r="W9" s="12"/>
     </row>
-    <row r="10" spans="1:23" ht="40" customHeight="1">
+    <row r="10" spans="1:23" ht="56" customHeight="1">
       <c r="A10" s="15" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="E10" s="15" t="s">
         <v>149</v>
@@ -3532,7 +3607,7 @@
     </row>
     <row r="3" spans="1:21" ht="30" customHeight="1" thickTop="1">
       <c r="A3" s="5" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>132</v>
@@ -3552,27 +3627,27 @@
     </row>
     <row r="4" spans="1:21" s="16" customFormat="1" ht="46" customHeight="1">
       <c r="A4" s="19" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B4" s="19" t="s">
+        <v>198</v>
+      </c>
+      <c r="C4" s="19" t="s">
+        <v>199</v>
+      </c>
+      <c r="D4" s="19" t="s">
         <v>200</v>
-      </c>
-      <c r="C4" s="19" t="s">
-        <v>201</v>
-      </c>
-      <c r="D4" s="19" t="s">
-        <v>202</v>
       </c>
       <c r="E4" s="19" t="s">
         <v>174</v>
       </c>
       <c r="F4" s="20" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
     </row>
     <row r="5" spans="1:21" s="16" customFormat="1" ht="50" customHeight="1">
       <c r="A5" s="19" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B5" s="19" t="s">
         <v>166</v>
@@ -3607,7 +3682,7 @@
     </row>
     <row r="6" spans="1:21" s="16" customFormat="1" ht="50" customHeight="1">
       <c r="A6" s="19" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B6" s="19" t="s">
         <v>180</v>
@@ -3616,13 +3691,13 @@
         <v>181</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>183</v>
+        <v>244</v>
       </c>
       <c r="E6" s="19" t="s">
         <v>173</v>
       </c>
       <c r="F6" s="20" t="s">
-        <v>184</v>
+        <v>245</v>
       </c>
       <c r="G6" s="17"/>
       <c r="H6" s="17"/>
@@ -3642,7 +3717,7 @@
     </row>
     <row r="7" spans="1:21" s="16" customFormat="1" ht="50" customHeight="1">
       <c r="A7" s="19" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B7" s="20" t="s">
         <v>167</v>
@@ -3677,7 +3752,7 @@
     </row>
     <row r="8" spans="1:21" s="16" customFormat="1" ht="50" customHeight="1">
       <c r="A8" s="19" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B8" s="20" t="s">
         <v>168</v>
@@ -3712,7 +3787,7 @@
     </row>
     <row r="9" spans="1:21" s="16" customFormat="1" ht="50" customHeight="1">
       <c r="A9" s="19" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B9" s="20" t="s">
         <v>169</v>
@@ -3747,7 +3822,7 @@
     </row>
     <row r="10" spans="1:21" s="16" customFormat="1" ht="50" customHeight="1">
       <c r="A10" s="19" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B10" s="20" t="s">
         <v>170</v>
@@ -3782,7 +3857,7 @@
     </row>
     <row r="11" spans="1:21" s="16" customFormat="1" ht="50" customHeight="1">
       <c r="A11" s="19" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B11" s="20" t="s">
         <v>171</v>
@@ -3817,16 +3892,16 @@
     </row>
     <row r="12" spans="1:21" s="16" customFormat="1" ht="50" customHeight="1">
       <c r="A12" s="19" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B12" s="20" t="s">
+        <v>188</v>
+      </c>
+      <c r="C12" s="20" t="s">
+        <v>189</v>
+      </c>
+      <c r="D12" s="19" t="s">
         <v>190</v>
-      </c>
-      <c r="C12" s="20" t="s">
-        <v>191</v>
-      </c>
-      <c r="D12" s="19" t="s">
-        <v>192</v>
       </c>
       <c r="E12" s="19" t="s">
         <v>175</v>
@@ -3852,16 +3927,16 @@
     </row>
     <row r="13" spans="1:21" s="16" customFormat="1" ht="50" customHeight="1">
       <c r="A13" s="19" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B13" s="20" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C13" s="20" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="E13" s="19" t="s">
         <v>173</v>
@@ -3887,22 +3962,22 @@
     </row>
     <row r="14" spans="1:21" s="16" customFormat="1" ht="84" customHeight="1">
       <c r="A14" s="19" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B14" s="20" t="s">
+        <v>192</v>
+      </c>
+      <c r="C14" s="20" t="s">
+        <v>193</v>
+      </c>
+      <c r="D14" s="19" t="s">
         <v>194</v>
-      </c>
-      <c r="C14" s="20" t="s">
-        <v>195</v>
-      </c>
-      <c r="D14" s="19" t="s">
-        <v>196</v>
       </c>
       <c r="E14" s="19" t="s">
         <v>175</v>
       </c>
       <c r="F14" s="19" t="s">
-        <v>185</v>
+        <v>246</v>
       </c>
       <c r="G14" s="17"/>
       <c r="H14" s="17"/>
@@ -3922,16 +3997,16 @@
     </row>
     <row r="15" spans="1:21" s="16" customFormat="1" ht="84" customHeight="1">
       <c r="A15" s="19" t="s">
+        <v>211</v>
+      </c>
+      <c r="B15" s="20" t="s">
+        <v>212</v>
+      </c>
+      <c r="C15" s="20" t="s">
         <v>214</v>
       </c>
-      <c r="B15" s="20" t="s">
-        <v>215</v>
-      </c>
-      <c r="C15" s="20" t="s">
-        <v>217</v>
-      </c>
       <c r="D15" s="19" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="E15" s="19"/>
       <c r="F15" s="19"/>
@@ -3953,16 +4028,16 @@
     </row>
     <row r="16" spans="1:21" s="16" customFormat="1" ht="84" customHeight="1">
       <c r="A16" s="19" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B16" s="20" t="s">
+        <v>213</v>
+      </c>
+      <c r="C16" s="20" t="s">
+        <v>215</v>
+      </c>
+      <c r="D16" s="19" t="s">
         <v>216</v>
-      </c>
-      <c r="C16" s="20" t="s">
-        <v>218</v>
-      </c>
-      <c r="D16" s="19" t="s">
-        <v>219</v>
       </c>
       <c r="E16" s="19"/>
       <c r="F16" s="19"/>
@@ -3984,7 +4059,7 @@
     </row>
     <row r="17" spans="1:21" s="16" customFormat="1" ht="50" customHeight="1">
       <c r="A17" s="19" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B17" s="19" t="s">
         <v>172</v>
@@ -3999,7 +4074,7 @@
         <v>173</v>
       </c>
       <c r="F17" s="19" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="G17" s="17"/>
       <c r="H17" s="17"/>
@@ -4019,22 +4094,22 @@
     </row>
     <row r="18" spans="1:21" s="16" customFormat="1" ht="50" customHeight="1">
       <c r="A18" s="19" t="s">
+        <v>219</v>
+      </c>
+      <c r="B18" s="21" t="s">
         <v>222</v>
       </c>
-      <c r="B18" s="21" t="s">
-        <v>225</v>
-      </c>
       <c r="C18" s="19" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="D18" s="19" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="E18" s="19" t="s">
         <v>174</v>
       </c>
       <c r="F18" s="19" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="G18" s="17"/>
       <c r="H18" s="17"/>
@@ -4054,7 +4129,7 @@
     </row>
     <row r="19" spans="1:21" s="16" customFormat="1" ht="50" customHeight="1">
       <c r="A19" s="19" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="B19" s="21" t="s">
         <v>166</v>
@@ -4069,7 +4144,7 @@
         <v>173</v>
       </c>
       <c r="F19" s="19" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="G19" s="17"/>
       <c r="H19" s="17"/>
@@ -4089,16 +4164,16 @@
     </row>
     <row r="20" spans="1:21" s="16" customFormat="1" ht="50" customHeight="1">
       <c r="A20" s="19" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="B20" s="21" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="C20" s="19" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="E20" s="19" t="s">
         <v>173</v>
@@ -4124,16 +4199,16 @@
     </row>
     <row r="21" spans="1:21" s="16" customFormat="1" ht="50" customHeight="1">
       <c r="A21" s="19" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="B21" s="21" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E21" s="19" t="s">
         <v>173</v>
@@ -4157,24 +4232,24 @@
       <c r="T21" s="18"/>
       <c r="U21" s="18"/>
     </row>
-    <row r="22" spans="1:21" s="16" customFormat="1" ht="50" customHeight="1">
+    <row r="22" spans="1:21" s="16" customFormat="1" ht="73" customHeight="1">
       <c r="A22" s="19" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="B22" s="21" t="s">
+        <v>192</v>
+      </c>
+      <c r="C22" s="19" t="s">
+        <v>193</v>
+      </c>
+      <c r="D22" s="19" t="s">
         <v>194</v>
-      </c>
-      <c r="C22" s="19" t="s">
-        <v>195</v>
-      </c>
-      <c r="D22" s="19" t="s">
-        <v>196</v>
       </c>
       <c r="E22" s="19" t="s">
         <v>175</v>
       </c>
       <c r="F22" s="19" t="s">
-        <v>185</v>
+        <v>246</v>
       </c>
       <c r="G22" s="18"/>
       <c r="H22" s="18"/>
@@ -4194,16 +4269,16 @@
     </row>
     <row r="23" spans="1:21" s="16" customFormat="1" ht="50" customHeight="1">
       <c r="A23" s="19" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="B23" s="21" t="s">
+        <v>188</v>
+      </c>
+      <c r="C23" s="19" t="s">
+        <v>189</v>
+      </c>
+      <c r="D23" s="19" t="s">
         <v>190</v>
-      </c>
-      <c r="C23" s="19" t="s">
-        <v>191</v>
-      </c>
-      <c r="D23" s="19" t="s">
-        <v>192</v>
       </c>
       <c r="E23" s="19" t="s">
         <v>175</v>
@@ -4229,16 +4304,16 @@
     </row>
     <row r="24" spans="1:21" s="16" customFormat="1" ht="50" customHeight="1">
       <c r="A24" s="19" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D24" s="19" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="E24" s="19" t="s">
         <v>173</v>
@@ -4264,22 +4339,22 @@
     </row>
     <row r="25" spans="1:21" s="16" customFormat="1" ht="50" customHeight="1">
       <c r="A25" s="19" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="B25" s="21" t="s">
+        <v>225</v>
+      </c>
+      <c r="C25" s="19" t="s">
         <v>228</v>
       </c>
-      <c r="C25" s="19" t="s">
+      <c r="D25" s="19" t="s">
         <v>231</v>
-      </c>
-      <c r="D25" s="19" t="s">
-        <v>234</v>
       </c>
       <c r="E25" s="19" t="s">
         <v>173</v>
       </c>
       <c r="F25" s="19" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="G25" s="18"/>
       <c r="H25" s="18"/>
@@ -5647,16 +5722,16 @@
     </row>
     <row r="4" spans="1:19" ht="50" customHeight="1">
       <c r="A4" s="31" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B4" s="31" t="s">
         <v>156</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="D4" s="31" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="E4" s="31"/>
       <c r="F4" s="24"/>
@@ -7690,14 +7765,14 @@
         <v>177</v>
       </c>
       <c r="B4" s="28" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C4" s="28"/>
       <c r="D4" s="28" t="s">
         <v>178</v>
       </c>
       <c r="E4" s="28" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="F4" s="12"/>
       <c r="G4" s="12"/>
@@ -7719,14 +7794,14 @@
         <v>179</v>
       </c>
       <c r="B5" s="30" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C5" s="28"/>
       <c r="D5" s="28" t="s">
         <v>178</v>
       </c>
       <c r="E5" s="28" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="F5" s="12"/>
       <c r="G5" s="12"/>
@@ -7745,17 +7820,17 @@
     </row>
     <row r="6" spans="1:19" ht="50" customHeight="1">
       <c r="A6" s="29" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B6" s="30" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C6" s="28"/>
       <c r="D6" s="28" t="s">
         <v>178</v>
       </c>
       <c r="E6" s="28" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="F6" s="12"/>
       <c r="G6" s="12"/>
@@ -7774,17 +7849,17 @@
     </row>
     <row r="7" spans="1:19" ht="50" customHeight="1">
       <c r="A7" s="29" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B7" s="30" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C7" s="28"/>
       <c r="D7" s="28" t="s">
         <v>178</v>
       </c>
       <c r="E7" s="28" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="F7" s="12"/>
       <c r="G7" s="12"/>
@@ -7803,17 +7878,17 @@
     </row>
     <row r="8" spans="1:19" ht="50" customHeight="1">
       <c r="A8" s="29" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B8" s="30" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C8" s="28"/>
       <c r="D8" s="28" t="s">
         <v>178</v>
       </c>
       <c r="E8" s="28" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="F8" s="12"/>
       <c r="G8" s="12"/>
@@ -7832,17 +7907,17 @@
     </row>
     <row r="9" spans="1:19" ht="50" customHeight="1">
       <c r="A9" s="29" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="B9" s="30" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C9" s="28"/>
       <c r="D9" s="28" t="s">
         <v>178</v>
       </c>
       <c r="E9" s="28" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="F9" s="12"/>
       <c r="G9" s="12"/>
@@ -7860,11 +7935,19 @@
       <c r="S9" s="12"/>
     </row>
     <row r="10" spans="1:19" ht="50" customHeight="1">
-      <c r="A10" s="13"/>
-      <c r="B10" s="13"/>
-      <c r="C10" s="12"/>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12"/>
+      <c r="A10" s="29" t="s">
+        <v>242</v>
+      </c>
+      <c r="B10" s="30" t="s">
+        <v>243</v>
+      </c>
+      <c r="C10" s="28"/>
+      <c r="D10" s="28" t="s">
+        <v>178</v>
+      </c>
+      <c r="E10" s="28" t="s">
+        <v>204</v>
+      </c>
       <c r="F10" s="12"/>
       <c r="G10" s="12"/>
       <c r="H10" s="12"/>

</xml_diff>